<commit_message>
feat: Update marka_new.json to add new vehicle brands and enhance catalog information
</commit_message>
<xml_diff>
--- a/src/output/Drum/excels/OE/Drum_OE_Numbers_full.xlsx
+++ b/src/output/Drum/excels/OE/Drum_OE_Numbers_full.xlsx
@@ -8,17 +8,14 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\URETIM9\Desktop\Projects\API_SCRAPE\src\output\Drum\excels\OE\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F26A38AF-3440-4C4F-B3B9-2313B42B8EB4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{78E43BF3-81DD-4D0E-91BB-3881AD7FA115}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-15240" yWindow="396" windowWidth="20532" windowHeight="10140" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="804" yWindow="2220" windowWidth="20532" windowHeight="10140" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="OE_Numbers" sheetId="1" r:id="rId1"/>
     <sheet name="BULUNAMAYANLAR" sheetId="2" r:id="rId2"/>
   </sheets>
-  <externalReferences>
-    <externalReference r:id="rId3"/>
-  </externalReferences>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">BULUNAMAYANLAR!$A$1:$C$118</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">OE_Numbers!$A$1:$E$474</definedName>
@@ -39,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2345" uniqueCount="679">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2359" uniqueCount="691">
   <si>
     <t>YV</t>
   </si>
@@ -2076,6 +2073,42 @@
   </si>
   <si>
     <t>8944766711</t>
+  </si>
+  <si>
+    <t>043860</t>
+  </si>
+  <si>
+    <t>HST1126AB</t>
+  </si>
+  <si>
+    <t>90PY1126</t>
+  </si>
+  <si>
+    <t>3757089</t>
+  </si>
+  <si>
+    <t>28288</t>
+  </si>
+  <si>
+    <t>2952956</t>
+  </si>
+  <si>
+    <t>57RS305352</t>
+  </si>
+  <si>
+    <t>3302350207001</t>
+  </si>
+  <si>
+    <t>MC862229</t>
+  </si>
+  <si>
+    <t>8941010571</t>
+  </si>
+  <si>
+    <t>8973341070AA</t>
+  </si>
+  <si>
+    <t>R2X61126AAN</t>
   </si>
 </sst>
 </file>
@@ -2166,3447 +2199,6 @@
     </ext>
   </extLst>
 </styleSheet>
-</file>
-
-<file path=xl/externalLinks/externalLink1.xml><?xml version="1.0" encoding="utf-8"?>
-<externalLink xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" mc:Ignorable="x14">
-  <externalBook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1">
-    <sheetNames>
-      <sheetName val="Sheet1"/>
-      <sheetName val="BULUNAMAYANLAR"/>
-    </sheetNames>
-    <sheetDataSet>
-      <sheetData sheetId="0">
-        <row r="1">
-          <cell r="A1" t="str">
-            <v>YV</v>
-          </cell>
-          <cell r="B1" t="str">
-            <v>BREMBO</v>
-          </cell>
-          <cell r="C1" t="str">
-            <v>TRW</v>
-          </cell>
-          <cell r="D1" t="str">
-            <v>Delphi  No</v>
-          </cell>
-          <cell r="E1" t="str">
-            <v>Ferodo No</v>
-          </cell>
-          <cell r="F1" t="str">
-            <v>FREMAX</v>
-          </cell>
-          <cell r="G1" t="str">
-            <v>ICER No</v>
-          </cell>
-          <cell r="H1" t="str">
-            <v>BOSCH</v>
-          </cell>
-          <cell r="I1" t="str">
-            <v>NK</v>
-          </cell>
-          <cell r="J1" t="str">
-            <v>Optimal no</v>
-          </cell>
-          <cell r="K1" t="str">
-            <v>BRAXIS</v>
-          </cell>
-          <cell r="L1" t="str">
-            <v>KRAFTVOLL</v>
-          </cell>
-          <cell r="M1" t="str">
-            <v>KRAFTVOLL</v>
-          </cell>
-          <cell r="N1" t="str">
-            <v>kale no</v>
-          </cell>
-          <cell r="O1" t="str">
-            <v>Netex no</v>
-          </cell>
-          <cell r="P1" t="str">
-            <v>RAION stok kodu</v>
-          </cell>
-          <cell r="Q1" t="str">
-            <v>BSG</v>
-          </cell>
-          <cell r="R1" t="str">
-            <v>TEXTAR</v>
-          </cell>
-          <cell r="S1" t="str">
-            <v>JNBK</v>
-          </cell>
-          <cell r="T1" t="str">
-            <v>OE_1</v>
-          </cell>
-        </row>
-        <row r="2">
-          <cell r="A2">
-            <v>24163</v>
-          </cell>
-          <cell r="B2" t="str">
-            <v>14.3260.10</v>
-          </cell>
-          <cell r="C2" t="str">
-            <v>DB4038</v>
-          </cell>
-          <cell r="D2" t="str">
-            <v>BF168</v>
-          </cell>
-          <cell r="N2" t="str">
-            <v>TFD-00420</v>
-          </cell>
-          <cell r="Q2" t="str">
-            <v>BSG 60-225-001</v>
-          </cell>
-          <cell r="T2" t="str">
-            <v>6014235101</v>
-          </cell>
-        </row>
-        <row r="3">
-          <cell r="A3">
-            <v>24165</v>
-          </cell>
-          <cell r="B3" t="str">
-            <v>14.5603.10</v>
-          </cell>
-          <cell r="C3" t="str">
-            <v>DB4089</v>
-          </cell>
-          <cell r="N3" t="str">
-            <v>TFD-00422</v>
-          </cell>
-          <cell r="Q3" t="str">
-            <v>BSG 60-225-002</v>
-          </cell>
-          <cell r="T3" t="str">
-            <v>6014235001</v>
-          </cell>
-        </row>
-        <row r="4">
-          <cell r="A4">
-            <v>13275</v>
-          </cell>
-          <cell r="L4" t="str">
-            <v>07050077</v>
-          </cell>
-          <cell r="M4"/>
-          <cell r="N4" t="str">
-            <v>TFD-00359</v>
-          </cell>
-          <cell r="T4" t="str">
-            <v>043860</v>
-          </cell>
-        </row>
-        <row r="5">
-          <cell r="A5">
-            <v>13277</v>
-          </cell>
-          <cell r="B5" t="str">
-            <v>14.3166.10</v>
-          </cell>
-          <cell r="C5" t="str">
-            <v>DB4004</v>
-          </cell>
-          <cell r="D5" t="str">
-            <v>BF107</v>
-          </cell>
-          <cell r="J5" t="str">
-            <v>BT-0340</v>
-          </cell>
-          <cell r="L5" t="str">
-            <v>07050078</v>
-          </cell>
-          <cell r="M5" t="str">
-            <v>07050078</v>
-          </cell>
-          <cell r="N5" t="str">
-            <v>TFD-00360</v>
-          </cell>
-          <cell r="Q5" t="str">
-            <v>BSG 30-225-022</v>
-          </cell>
-          <cell r="T5" t="str">
-            <v>6046462</v>
-          </cell>
-        </row>
-        <row r="6">
-          <cell r="A6">
-            <v>13278</v>
-          </cell>
-          <cell r="L6" t="str">
-            <v>07050079</v>
-          </cell>
-          <cell r="M6"/>
-          <cell r="N6" t="str">
-            <v>TFD-00361</v>
-          </cell>
-          <cell r="T6" t="str">
-            <v>HST1126AB</v>
-          </cell>
-        </row>
-        <row r="7">
-          <cell r="A7">
-            <v>13279</v>
-          </cell>
-          <cell r="B7" t="str">
-            <v>14.6794.10</v>
-          </cell>
-          <cell r="C7" t="str">
-            <v>DB4041</v>
-          </cell>
-          <cell r="L7" t="str">
-            <v>07050080</v>
-          </cell>
-          <cell r="M7" t="str">
-            <v>07050080</v>
-          </cell>
-          <cell r="N7" t="str">
-            <v>TFD-00362</v>
-          </cell>
-          <cell r="Q7" t="str">
-            <v>BSG 30-225-023</v>
-          </cell>
-          <cell r="T7" t="str">
-            <v>6008179</v>
-          </cell>
-        </row>
-        <row r="8">
-          <cell r="A8">
-            <v>13280</v>
-          </cell>
-          <cell r="B8" t="str">
-            <v>14.6795.10</v>
-          </cell>
-          <cell r="L8" t="str">
-            <v>07050081</v>
-          </cell>
-          <cell r="M8"/>
-          <cell r="N8" t="str">
-            <v>TFD-00363</v>
-          </cell>
-          <cell r="T8" t="str">
-            <v>6049432</v>
-          </cell>
-        </row>
-        <row r="9">
-          <cell r="A9">
-            <v>13281</v>
-          </cell>
-          <cell r="B9" t="str">
-            <v>14.7099.10</v>
-          </cell>
-          <cell r="C9" t="str">
-            <v>DB4167</v>
-          </cell>
-          <cell r="D9" t="str">
-            <v>BF317</v>
-          </cell>
-          <cell r="J9" t="str">
-            <v>BT-0800</v>
-          </cell>
-          <cell r="K9" t="str">
-            <v>AD5022</v>
-          </cell>
-          <cell r="L9" t="str">
-            <v>07050012</v>
-          </cell>
-          <cell r="M9" t="str">
-            <v>07050012</v>
-          </cell>
-          <cell r="N9" t="str">
-            <v>TFD-00364</v>
-          </cell>
-          <cell r="Q9" t="str">
-            <v>BSG 30-225-002</v>
-          </cell>
-          <cell r="T9" t="str">
-            <v>92VB1126BA</v>
-          </cell>
-        </row>
-        <row r="10">
-          <cell r="A10">
-            <v>13282</v>
-          </cell>
-          <cell r="B10" t="str">
-            <v>14.7098.10</v>
-          </cell>
-          <cell r="C10" t="str">
-            <v>DB4166</v>
-          </cell>
-          <cell r="D10" t="str">
-            <v>BF316</v>
-          </cell>
-          <cell r="J10" t="str">
-            <v>BT-1380</v>
-          </cell>
-          <cell r="K10" t="str">
-            <v>AD5021</v>
-          </cell>
-          <cell r="L10" t="str">
-            <v>07050014</v>
-          </cell>
-          <cell r="M10" t="str">
-            <v>07050014</v>
-          </cell>
-          <cell r="N10" t="str">
-            <v>TFD-00365</v>
-          </cell>
-          <cell r="Q10" t="str">
-            <v>BSG 30-225-001</v>
-          </cell>
-          <cell r="T10" t="str">
-            <v>92VB1126AA</v>
-          </cell>
-        </row>
-        <row r="11">
-          <cell r="A11">
-            <v>13283</v>
-          </cell>
-          <cell r="B11" t="str">
-            <v>14.7008.10, 14.7247.10</v>
-          </cell>
-          <cell r="C11" t="str">
-            <v>DB4156</v>
-          </cell>
-          <cell r="F11" t="str">
-            <v>BD-6630</v>
-          </cell>
-          <cell r="K11" t="str">
-            <v>AD5112</v>
-          </cell>
-          <cell r="L11" t="str">
-            <v>07050082</v>
-          </cell>
-          <cell r="M11" t="str">
-            <v>07050082</v>
-          </cell>
-          <cell r="N11" t="str">
-            <v>TFD-00366</v>
-          </cell>
-          <cell r="Q11" t="str">
-            <v>BSG 30-225-024</v>
-          </cell>
-          <cell r="T11" t="str">
-            <v>96AA111395</v>
-          </cell>
-        </row>
-        <row r="12">
-          <cell r="A12">
-            <v>13284</v>
-          </cell>
-          <cell r="L12" t="str">
-            <v>07050083</v>
-          </cell>
-          <cell r="M12"/>
-          <cell r="N12" t="str">
-            <v>TFD-00367</v>
-          </cell>
-          <cell r="T12" t="str">
-            <v>90PY1126</v>
-          </cell>
-        </row>
-        <row r="13">
-          <cell r="A13">
-            <v>13285</v>
-          </cell>
-          <cell r="B13" t="str">
-            <v>14.A692.10</v>
-          </cell>
-          <cell r="C13" t="str">
-            <v>DB4316</v>
-          </cell>
-          <cell r="D13" t="str">
-            <v>BF478</v>
-          </cell>
-          <cell r="J13" t="str">
-            <v>BT-1980</v>
-          </cell>
-          <cell r="K13" t="str">
-            <v>AD5020</v>
-          </cell>
-          <cell r="L13" t="str">
-            <v>07050015</v>
-          </cell>
-          <cell r="M13" t="str">
-            <v>07050015</v>
-          </cell>
-          <cell r="N13" t="str">
-            <v>TFD-00368</v>
-          </cell>
-          <cell r="Q13" t="str">
-            <v>BSG 30-225-003</v>
-          </cell>
-          <cell r="R13" t="str">
-            <v>94024600</v>
-          </cell>
-          <cell r="S13"/>
-          <cell r="T13" t="str">
-            <v>4078769</v>
-          </cell>
-        </row>
-        <row r="14">
-          <cell r="A14">
-            <v>13286</v>
-          </cell>
-          <cell r="B14" t="str">
-            <v>14.A693.10</v>
-          </cell>
-          <cell r="C14" t="str">
-            <v>DB4315</v>
-          </cell>
-          <cell r="D14" t="str">
-            <v>BF467</v>
-          </cell>
-          <cell r="K14" t="str">
-            <v>AD5019</v>
-          </cell>
-          <cell r="L14" t="str">
-            <v>07050026</v>
-          </cell>
-          <cell r="M14" t="str">
-            <v>07050026</v>
-          </cell>
-          <cell r="N14" t="str">
-            <v>TFD-00369</v>
-          </cell>
-          <cell r="R14" t="str">
-            <v>94024800</v>
-          </cell>
-          <cell r="S14"/>
-          <cell r="T14" t="str">
-            <v>YC1W1126ED</v>
-          </cell>
-        </row>
-        <row r="15">
-          <cell r="A15">
-            <v>13290</v>
-          </cell>
-          <cell r="B15" t="str">
-            <v>14.A691.10</v>
-          </cell>
-          <cell r="C15" t="str">
-            <v>DB4309</v>
-          </cell>
-          <cell r="D15" t="str">
-            <v>BF488</v>
-          </cell>
-          <cell r="K15" t="str">
-            <v>AD5017</v>
-          </cell>
-          <cell r="L15" t="str">
-            <v>07050010</v>
-          </cell>
-          <cell r="M15" t="str">
-            <v>07050010</v>
-          </cell>
-          <cell r="N15" t="str">
-            <v>TFD-00371</v>
-          </cell>
-          <cell r="R15" t="str">
-            <v>94024400</v>
-          </cell>
-          <cell r="S15"/>
-          <cell r="T15" t="str">
-            <v>4467600</v>
-          </cell>
-        </row>
-        <row r="16">
-          <cell r="A16">
-            <v>13289</v>
-          </cell>
-          <cell r="C16" t="str">
-            <v>DB4338B</v>
-          </cell>
-          <cell r="K16" t="str">
-            <v>AD5018</v>
-          </cell>
-          <cell r="L16" t="str">
-            <v>07050017</v>
-          </cell>
-          <cell r="M16" t="str">
-            <v>07050017</v>
-          </cell>
-          <cell r="N16" t="str">
-            <v>TFD-00370</v>
-          </cell>
-          <cell r="R16" t="str">
-            <v>94022500</v>
-          </cell>
-          <cell r="S16"/>
-          <cell r="T16" t="str">
-            <v>1M5W1113AA</v>
-          </cell>
-        </row>
-        <row r="17">
-          <cell r="A17">
-            <v>36020</v>
-          </cell>
-          <cell r="B17" t="str">
-            <v>14.3256.10</v>
-          </cell>
-          <cell r="C17" t="str">
-            <v>DB4081</v>
-          </cell>
-          <cell r="D17" t="str">
-            <v>BF96</v>
-          </cell>
-          <cell r="E17" t="str">
-            <v>FDR329128</v>
-          </cell>
-          <cell r="F17" t="str">
-            <v>BD-1511</v>
-          </cell>
-          <cell r="J17" t="str">
-            <v>BT-0070</v>
-          </cell>
-          <cell r="K17" t="str">
-            <v>AD5027</v>
-          </cell>
-          <cell r="L17" t="str">
-            <v>07050029</v>
-          </cell>
-          <cell r="M17" t="str">
-            <v>07050029</v>
-          </cell>
-          <cell r="N17" t="str">
-            <v>TFD-00593</v>
-          </cell>
-          <cell r="O17" t="str">
-            <v>BD200 4081</v>
-          </cell>
-          <cell r="P17" t="str">
-            <v xml:space="preserve">191-501-615B/RAION
-</v>
-          </cell>
-          <cell r="Q17" t="str">
-            <v>BSG 90-225-002</v>
-          </cell>
-          <cell r="R17" t="str">
-            <v>94006600</v>
-          </cell>
-          <cell r="S17"/>
-          <cell r="T17" t="str">
-            <v>171501615</v>
-          </cell>
-        </row>
-        <row r="18">
-          <cell r="A18">
-            <v>25181</v>
-          </cell>
-          <cell r="C18" t="str">
-            <v>DB4313</v>
-          </cell>
-          <cell r="J18" t="str">
-            <v>BT-2010</v>
-          </cell>
-          <cell r="K18" t="str">
-            <v>AD5011</v>
-          </cell>
-          <cell r="L18" t="str">
-            <v>07050018</v>
-          </cell>
-          <cell r="M18" t="str">
-            <v>07050018</v>
-          </cell>
-          <cell r="N18" t="str">
-            <v>TFD-00448</v>
-          </cell>
-          <cell r="P18" t="str">
-            <v>RAI-KD02008</v>
-          </cell>
-          <cell r="Q18" t="str">
-            <v>BSG 62-225-003</v>
-          </cell>
-          <cell r="T18" t="str">
-            <v>MB193595</v>
-          </cell>
-        </row>
-        <row r="19">
-          <cell r="A19">
-            <v>18160</v>
-          </cell>
-          <cell r="C19" t="str">
-            <v>DB4449</v>
-          </cell>
-          <cell r="K19" t="str">
-            <v>AD5012</v>
-          </cell>
-          <cell r="L19" t="str">
-            <v>07050003</v>
-          </cell>
-          <cell r="M19" t="str">
-            <v>07050003</v>
-          </cell>
-          <cell r="N19" t="str">
-            <v>TFD-00390</v>
-          </cell>
-          <cell r="O19" t="str">
-            <v>BD200 4449</v>
-          </cell>
-          <cell r="P19" t="str">
-            <v>RAI-KD02005</v>
-          </cell>
-          <cell r="Q19" t="str">
-            <v>BSG 40-225-007</v>
-          </cell>
-          <cell r="T19" t="str">
-            <v>0K60B26251</v>
-          </cell>
-        </row>
-        <row r="20">
-          <cell r="A20">
-            <v>16183</v>
-          </cell>
-          <cell r="C20" t="str">
-            <v>DB4377</v>
-          </cell>
-          <cell r="K20" t="str">
-            <v>AD5015</v>
-          </cell>
-          <cell r="L20" t="str">
-            <v>07050002</v>
-          </cell>
-          <cell r="M20" t="str">
-            <v>07050002</v>
-          </cell>
-          <cell r="N20" t="str">
-            <v>TFD-00384</v>
-          </cell>
-          <cell r="P20" t="str">
-            <v>RAI-KD02001</v>
-          </cell>
-          <cell r="Q20" t="str">
-            <v>BSG 40-225-006</v>
-          </cell>
-          <cell r="T20" t="str">
-            <v>5276144102</v>
-          </cell>
-        </row>
-        <row r="21">
-          <cell r="A21">
-            <v>33149</v>
-          </cell>
-          <cell r="B21" t="str">
-            <v>14.7076.10</v>
-          </cell>
-          <cell r="C21" t="str">
-            <v>DB4162</v>
-          </cell>
-          <cell r="D21" t="str">
-            <v>BF327</v>
-          </cell>
-          <cell r="E21" t="str">
-            <v>FDR329011</v>
-          </cell>
-          <cell r="J21" t="str">
-            <v>BT-2230</v>
-          </cell>
-          <cell r="K21" t="str">
-            <v>AD5003</v>
-          </cell>
-          <cell r="L21" t="str">
-            <v>07050011</v>
-          </cell>
-          <cell r="M21" t="str">
-            <v>07050011</v>
-          </cell>
-          <cell r="N21" t="str">
-            <v>TFD-00579</v>
-          </cell>
-          <cell r="O21" t="str">
-            <v>BD200 4162</v>
-          </cell>
-          <cell r="R21" t="str">
-            <v>94014600</v>
-          </cell>
-          <cell r="S21"/>
-          <cell r="T21" t="str">
-            <v>424738</v>
-          </cell>
-        </row>
-        <row r="22">
-          <cell r="A22">
-            <v>40217</v>
-          </cell>
-          <cell r="B22" t="str">
-            <v>14.4733.10</v>
-          </cell>
-          <cell r="C22" t="str">
-            <v>DB4136</v>
-          </cell>
-          <cell r="E22" t="str">
-            <v>FDR329213</v>
-          </cell>
-          <cell r="J22" t="str">
-            <v>BT-1320</v>
-          </cell>
-          <cell r="N22" t="str">
-            <v>TFD-00629</v>
-          </cell>
-          <cell r="P22" t="str">
-            <v>RAI-KD02007</v>
-          </cell>
-          <cell r="Q22" t="str">
-            <v>BSG 41-225-004</v>
-          </cell>
-          <cell r="T22" t="str">
-            <v>8942268291</v>
-          </cell>
-        </row>
-        <row r="23">
-          <cell r="A23">
-            <v>28324</v>
-          </cell>
-          <cell r="B23" t="str">
-            <v>14.3283.10</v>
-          </cell>
-          <cell r="C23" t="str">
-            <v>DB4096</v>
-          </cell>
-          <cell r="D23" t="str">
-            <v>BF169</v>
-          </cell>
-          <cell r="E23" t="str">
-            <v>DDF1212</v>
-          </cell>
-          <cell r="J23" t="str">
-            <v>BT-0320</v>
-          </cell>
-          <cell r="K23" t="str">
-            <v>AD5028</v>
-          </cell>
-          <cell r="L23" t="str">
-            <v>07050091</v>
-          </cell>
-          <cell r="M23" t="str">
-            <v>07050091</v>
-          </cell>
-          <cell r="N23" t="str">
-            <v>TFD-00516</v>
-          </cell>
-          <cell r="O23" t="str">
-            <v>BD200 4096</v>
-          </cell>
-          <cell r="R23" t="str">
-            <v>94010300</v>
-          </cell>
-          <cell r="S23"/>
-          <cell r="T23" t="str">
-            <v>424724</v>
-          </cell>
-        </row>
-        <row r="24">
-          <cell r="A24">
-            <v>36349</v>
-          </cell>
-          <cell r="C24" t="str">
-            <v>DB4143</v>
-          </cell>
-          <cell r="N24" t="str">
-            <v>TFD-00611</v>
-          </cell>
-          <cell r="Q24" t="str">
-            <v>BSG 90-225-003</v>
-          </cell>
-          <cell r="T24" t="str">
-            <v>113501615J</v>
-          </cell>
-        </row>
-        <row r="25">
-          <cell r="A25">
-            <v>40371</v>
-          </cell>
-          <cell r="B25" t="str">
-            <v>14.D629.10</v>
-          </cell>
-          <cell r="K25" t="str">
-            <v>AD5000</v>
-          </cell>
-          <cell r="L25" t="str">
-            <v>07050021</v>
-          </cell>
-          <cell r="M25" t="str">
-            <v>07050021</v>
-          </cell>
-          <cell r="N25" t="str">
-            <v>TFD-00631</v>
-          </cell>
-          <cell r="P25" t="str">
-            <v>RAI-KD02003</v>
-          </cell>
-          <cell r="Q25" t="str">
-            <v>BSG 41-225-001</v>
-          </cell>
-          <cell r="T25" t="str">
-            <v>8973605050</v>
-          </cell>
-        </row>
-        <row r="26">
-          <cell r="A26">
-            <v>40372</v>
-          </cell>
-          <cell r="B26" t="str">
-            <v>14.D630.10</v>
-          </cell>
-          <cell r="K26" t="str">
-            <v>AD5050</v>
-          </cell>
-          <cell r="L26" t="str">
-            <v>07050006</v>
-          </cell>
-          <cell r="M26" t="str">
-            <v>07050006</v>
-          </cell>
-          <cell r="N26" t="str">
-            <v>TFD-00632</v>
-          </cell>
-          <cell r="O26" t="str">
-            <v>BDK200 4451</v>
-          </cell>
-          <cell r="P26" t="str">
-            <v>RAI-KD02004</v>
-          </cell>
-          <cell r="Q26" t="str">
-            <v>BSG 41-225-002</v>
-          </cell>
-          <cell r="T26" t="str">
-            <v>8973605060</v>
-          </cell>
-        </row>
-        <row r="27">
-          <cell r="A27">
-            <v>27381</v>
-          </cell>
-          <cell r="B27" t="str">
-            <v>14.7715.10</v>
-          </cell>
-          <cell r="C27" t="str">
-            <v>DB4229</v>
-          </cell>
-          <cell r="D27" t="str">
-            <v>BF367</v>
-          </cell>
-          <cell r="E27" t="str">
-            <v>FDR329238</v>
-          </cell>
-          <cell r="F27" t="str">
-            <v>BD-8063</v>
-          </cell>
-          <cell r="L27" t="str">
-            <v>07050060</v>
-          </cell>
-          <cell r="M27" t="str">
-            <v>07050060</v>
-          </cell>
-          <cell r="N27" t="str">
-            <v>TFD-00488</v>
-          </cell>
-          <cell r="O27" t="str">
-            <v>BDK300 27381</v>
-          </cell>
-          <cell r="R27" t="str">
-            <v>94022600</v>
-          </cell>
-          <cell r="S27"/>
-          <cell r="T27" t="str">
-            <v>568063</v>
-          </cell>
-        </row>
-        <row r="28">
-          <cell r="A28">
-            <v>27382</v>
-          </cell>
-          <cell r="B28" t="str">
-            <v>14.4719.10</v>
-          </cell>
-          <cell r="C28" t="str">
-            <v>DB4002</v>
-          </cell>
-          <cell r="D28" t="str">
-            <v>BF102</v>
-          </cell>
-          <cell r="E28" t="str">
-            <v>FDR329202</v>
-          </cell>
-          <cell r="F28" t="str">
-            <v>BD-8958</v>
-          </cell>
-          <cell r="K28" t="str">
-            <v>AD5032</v>
-          </cell>
-          <cell r="L28" t="str">
-            <v>07050036</v>
-          </cell>
-          <cell r="M28" t="str">
-            <v>07050036</v>
-          </cell>
-          <cell r="N28" t="str">
-            <v>TFD-00489</v>
-          </cell>
-          <cell r="O28" t="str">
-            <v>BD200 4002</v>
-          </cell>
-          <cell r="Q28" t="str">
-            <v>BSG 65-225-002</v>
-          </cell>
-          <cell r="T28" t="str">
-            <v>568057</v>
-          </cell>
-        </row>
-        <row r="29">
-          <cell r="A29">
-            <v>27383</v>
-          </cell>
-          <cell r="B29" t="str">
-            <v>14.4718.10</v>
-          </cell>
-          <cell r="C29" t="str">
-            <v>DB4021</v>
-          </cell>
-          <cell r="D29" t="str">
-            <v>BF151</v>
-          </cell>
-          <cell r="E29" t="str">
-            <v>FDR329201</v>
-          </cell>
-          <cell r="K29" t="str">
-            <v>AD5009</v>
-          </cell>
-          <cell r="L29" t="str">
-            <v>07050013</v>
-          </cell>
-          <cell r="M29" t="str">
-            <v>07050013</v>
-          </cell>
-          <cell r="N29" t="str">
-            <v>TFD-00490</v>
-          </cell>
-          <cell r="O29" t="str">
-            <v>BD200 4021</v>
-          </cell>
-          <cell r="Q29" t="str">
-            <v>BSG 65-225-004</v>
-          </cell>
-          <cell r="T29" t="str">
-            <v>568058</v>
-          </cell>
-        </row>
-        <row r="30">
-          <cell r="A30">
-            <v>27384</v>
-          </cell>
-          <cell r="B30" t="str">
-            <v>14.4978.10</v>
-          </cell>
-          <cell r="C30" t="str">
-            <v>DB4006</v>
-          </cell>
-          <cell r="D30" t="str">
-            <v>BF111</v>
-          </cell>
-          <cell r="E30" t="str">
-            <v>FDR329711</v>
-          </cell>
-          <cell r="K30" t="str">
-            <v>AD5029</v>
-          </cell>
-          <cell r="L30" t="str">
-            <v>07050061</v>
-          </cell>
-          <cell r="M30" t="str">
-            <v>07050061</v>
-          </cell>
-          <cell r="N30" t="str">
-            <v>TFD-00491</v>
-          </cell>
-          <cell r="O30" t="str">
-            <v>BD200 4006</v>
-          </cell>
-          <cell r="Q30" t="str">
-            <v>BSG 65-210-005</v>
-          </cell>
-          <cell r="R30" t="str">
-            <v>94009900</v>
-          </cell>
-          <cell r="S30"/>
-          <cell r="T30" t="str">
-            <v>418117</v>
-          </cell>
-        </row>
-        <row r="31">
-          <cell r="A31">
-            <v>45387</v>
-          </cell>
-          <cell r="M31"/>
-          <cell r="N31" t="str">
-            <v>TFD-00682</v>
-          </cell>
-          <cell r="T31" t="str">
-            <v>3757089</v>
-          </cell>
-        </row>
-        <row r="32">
-          <cell r="A32">
-            <v>45396</v>
-          </cell>
-          <cell r="M32"/>
-          <cell r="N32" t="str">
-            <v>TFD-00683</v>
-          </cell>
-          <cell r="T32" t="str">
-            <v>28288</v>
-          </cell>
-        </row>
-        <row r="33">
-          <cell r="A33">
-            <v>25412</v>
-          </cell>
-          <cell r="B33" t="str">
-            <v>14.7096.10</v>
-          </cell>
-          <cell r="C33" t="str">
-            <v>DB4173</v>
-          </cell>
-          <cell r="D33" t="str">
-            <v>BF355</v>
-          </cell>
-          <cell r="J33" t="str">
-            <v>BT-0810</v>
-          </cell>
-          <cell r="K33" t="str">
-            <v>AD5010</v>
-          </cell>
-          <cell r="L33" t="str">
-            <v>07050016</v>
-          </cell>
-          <cell r="M33" t="str">
-            <v>07050016</v>
-          </cell>
-          <cell r="N33" t="str">
-            <v>TFD-00449</v>
-          </cell>
-          <cell r="O33" t="str">
-            <v>BD200 4173</v>
-          </cell>
-          <cell r="P33" t="str">
-            <v>RAI-KD02034</v>
-          </cell>
-          <cell r="Q33" t="str">
-            <v>BSG 62-225-001</v>
-          </cell>
-          <cell r="T33" t="str">
-            <v>MB950951</v>
-          </cell>
-        </row>
-        <row r="34">
-          <cell r="A34" t="str">
-            <v>45425H</v>
-          </cell>
-          <cell r="M34"/>
-          <cell r="N34" t="str">
-            <v>TFD-00685</v>
-          </cell>
-          <cell r="T34" t="str">
-            <v>2952956</v>
-          </cell>
-        </row>
-        <row r="35">
-          <cell r="A35">
-            <v>28431</v>
-          </cell>
-          <cell r="K35" t="str">
-            <v>AD5006</v>
-          </cell>
-          <cell r="L35" t="str">
-            <v>07050005</v>
-          </cell>
-          <cell r="M35" t="str">
-            <v>07050005</v>
-          </cell>
-          <cell r="N35" t="str">
-            <v>TFD-00523</v>
-          </cell>
-          <cell r="T35" t="str">
-            <v>P90005YP</v>
-          </cell>
-        </row>
-        <row r="36">
-          <cell r="A36">
-            <v>51435</v>
-          </cell>
-          <cell r="B36" t="str">
-            <v>14.A680.10</v>
-          </cell>
-          <cell r="N36" t="str">
-            <v>TFD-00721</v>
-          </cell>
-          <cell r="P36" t="str">
-            <v>RAI-KD02002</v>
-          </cell>
-          <cell r="T36" t="str">
-            <v>4243187602000</v>
-          </cell>
-        </row>
-        <row r="37">
-          <cell r="A37">
-            <v>27447</v>
-          </cell>
-          <cell r="B37" t="str">
-            <v>14.A694.10</v>
-          </cell>
-          <cell r="C37" t="str">
-            <v>DB4391</v>
-          </cell>
-          <cell r="E37" t="str">
-            <v>FDR329238</v>
-          </cell>
-          <cell r="K37" t="str">
-            <v>AD5008</v>
-          </cell>
-          <cell r="L37" t="str">
-            <v>07050001</v>
-          </cell>
-          <cell r="M37" t="str">
-            <v>07050001</v>
-          </cell>
-          <cell r="N37" t="str">
-            <v>TFD-00494</v>
-          </cell>
-          <cell r="O37" t="str">
-            <v>BDK300 27447</v>
-          </cell>
-          <cell r="Q37" t="str">
-            <v>BSG 65-210-030</v>
-          </cell>
-          <cell r="R37" t="str">
-            <v>94031500</v>
-          </cell>
-          <cell r="S37"/>
-          <cell r="T37" t="str">
-            <v>568066</v>
-          </cell>
-        </row>
-        <row r="38">
-          <cell r="A38">
-            <v>27448</v>
-          </cell>
-          <cell r="B38" t="str">
-            <v>14.A702.10</v>
-          </cell>
-          <cell r="C38" t="str">
-            <v>DB4301</v>
-          </cell>
-          <cell r="D38" t="str">
-            <v>BF471</v>
-          </cell>
-          <cell r="E38" t="str">
-            <v>FDR329713</v>
-          </cell>
-          <cell r="K38" t="str">
-            <v>AD5030</v>
-          </cell>
-          <cell r="L38" t="str">
-            <v>07050062</v>
-          </cell>
-          <cell r="M38" t="str">
-            <v>07050062</v>
-          </cell>
-          <cell r="N38" t="str">
-            <v>TFD-00495</v>
-          </cell>
-          <cell r="O38" t="str">
-            <v>BDK300 27448</v>
-          </cell>
-          <cell r="Q38" t="str">
-            <v>BSG 65-210-031</v>
-          </cell>
-          <cell r="R38" t="str">
-            <v>94024100</v>
-          </cell>
-          <cell r="S38"/>
-          <cell r="T38" t="str">
-            <v>418000</v>
-          </cell>
-        </row>
-        <row r="39">
-          <cell r="A39">
-            <v>18455</v>
-          </cell>
-          <cell r="F39"/>
-          <cell r="L39" t="str">
-            <v>07050025</v>
-          </cell>
-          <cell r="M39"/>
-          <cell r="N39" t="str">
-            <v>TFD-00397</v>
-          </cell>
-          <cell r="S39" t="str">
-            <v>DN1505</v>
-          </cell>
-          <cell r="T39" t="str">
-            <v>0K42A26251</v>
-          </cell>
-        </row>
-        <row r="40">
-          <cell r="A40">
-            <v>26463</v>
-          </cell>
-          <cell r="B40" t="str">
-            <v>14.6774.10</v>
-          </cell>
-          <cell r="K40" t="str">
-            <v>AD5035</v>
-          </cell>
-          <cell r="L40" t="str">
-            <v>07050024</v>
-          </cell>
-          <cell r="M40" t="str">
-            <v>07050024</v>
-          </cell>
-          <cell r="N40" t="str">
-            <v>TFD-00468</v>
-          </cell>
-          <cell r="P40" t="str">
-            <v>RAI-KD02032</v>
-          </cell>
-          <cell r="T40" t="str">
-            <v>4320631G11</v>
-          </cell>
-        </row>
-        <row r="41">
-          <cell r="A41">
-            <v>45473</v>
-          </cell>
-          <cell r="M41"/>
-          <cell r="N41" t="str">
-            <v>TFD-00688</v>
-          </cell>
-          <cell r="T41"/>
-        </row>
-        <row r="42">
-          <cell r="A42">
-            <v>59480</v>
-          </cell>
-          <cell r="K42" t="str">
-            <v>AD5048</v>
-          </cell>
-          <cell r="L42" t="str">
-            <v>07050030</v>
-          </cell>
-          <cell r="M42" t="str">
-            <v>07050030</v>
-          </cell>
-          <cell r="N42" t="str">
-            <v>TFD-00763</v>
-          </cell>
-          <cell r="T42" t="str">
-            <v>57RS305352</v>
-          </cell>
-        </row>
-        <row r="43">
-          <cell r="A43">
-            <v>27504</v>
-          </cell>
-          <cell r="B43" t="str">
-            <v>14.9390.10</v>
-          </cell>
-          <cell r="C43" t="str">
-            <v>DB4285</v>
-          </cell>
-          <cell r="D43" t="str">
-            <v>BF403</v>
-          </cell>
-          <cell r="E43" t="str">
-            <v>FDR329248</v>
-          </cell>
-          <cell r="K43" t="str">
-            <v>AD5007</v>
-          </cell>
-          <cell r="L43" t="str">
-            <v>07050019</v>
-          </cell>
-          <cell r="M43" t="str">
-            <v>07050019</v>
-          </cell>
-          <cell r="N43" t="str">
-            <v>TFD-00500</v>
-          </cell>
-          <cell r="O43" t="str">
-            <v>BD200 4285</v>
-          </cell>
-          <cell r="Q43" t="str">
-            <v>BSG 65-225-007</v>
-          </cell>
-          <cell r="T43" t="str">
-            <v>568060</v>
-          </cell>
-        </row>
-        <row r="44">
-          <cell r="A44">
-            <v>16508</v>
-          </cell>
-          <cell r="F44" t="str">
-            <v>BD-5131</v>
-          </cell>
-          <cell r="K44" t="str">
-            <v>AD5014</v>
-          </cell>
-          <cell r="L44" t="str">
-            <v>07050004</v>
-          </cell>
-          <cell r="M44" t="str">
-            <v>07050004</v>
-          </cell>
-          <cell r="N44" t="str">
-            <v>TFD-00385</v>
-          </cell>
-          <cell r="O44" t="str">
-            <v>BDK200 16508</v>
-          </cell>
-          <cell r="P44" t="str">
-            <v>RAI-KD02011</v>
-          </cell>
-          <cell r="Q44" t="str">
-            <v>BSG 40-225-001</v>
-          </cell>
-          <cell r="T44" t="str">
-            <v>584114F000</v>
-          </cell>
-        </row>
-        <row r="45">
-          <cell r="A45">
-            <v>25509</v>
-          </cell>
-          <cell r="C45" t="str">
-            <v>DB4423</v>
-          </cell>
-          <cell r="F45" t="str">
-            <v>BD-7020</v>
-          </cell>
-          <cell r="K45" t="str">
-            <v>AD5038</v>
-          </cell>
-          <cell r="L45" t="str">
-            <v>07040389</v>
-          </cell>
-          <cell r="M45" t="str">
-            <v>07040389</v>
-          </cell>
-          <cell r="N45" t="str">
-            <v>TFD-00452</v>
-          </cell>
-          <cell r="O45" t="str">
-            <v>BDK200 4423</v>
-          </cell>
-          <cell r="P45" t="str">
-            <v>RAI-KD02009</v>
-          </cell>
-          <cell r="Q45" t="str">
-            <v>BSG 62-225-002</v>
-          </cell>
-          <cell r="R45" t="str">
-            <v>94035300</v>
-          </cell>
-          <cell r="S45"/>
-          <cell r="T45" t="str">
-            <v>MN102439</v>
-          </cell>
-        </row>
-        <row r="46">
-          <cell r="A46">
-            <v>16518</v>
-          </cell>
-          <cell r="D46" t="str">
-            <v>BF520</v>
-          </cell>
-          <cell r="F46" t="str">
-            <v>BD-0101</v>
-          </cell>
-          <cell r="K46" t="str">
-            <v>AD5043</v>
-          </cell>
-          <cell r="L46" t="str">
-            <v>07040240</v>
-          </cell>
-          <cell r="M46" t="str">
-            <v>07040240</v>
-          </cell>
-          <cell r="N46" t="str">
-            <v>TFD-00386</v>
-          </cell>
-          <cell r="P46" t="str">
-            <v>RAI-KD02006</v>
-          </cell>
-          <cell r="Q46" t="str">
-            <v>BSG 40-225-002</v>
-          </cell>
-          <cell r="T46" t="str">
-            <v>5276144000</v>
-          </cell>
-        </row>
-        <row r="47">
-          <cell r="A47">
-            <v>59519</v>
-          </cell>
-          <cell r="K47" t="str">
-            <v>AD5059</v>
-          </cell>
-          <cell r="L47" t="str">
-            <v>07040370</v>
-          </cell>
-          <cell r="M47" t="str">
-            <v>07040370</v>
-          </cell>
-          <cell r="N47" t="str">
-            <v>TFD-00304</v>
-          </cell>
-          <cell r="T47" t="str">
-            <v>5M66346</v>
-          </cell>
-        </row>
-        <row r="48">
-          <cell r="A48">
-            <v>36532</v>
-          </cell>
-          <cell r="B48" t="str">
-            <v>14.9384.20</v>
-          </cell>
-          <cell r="C48" t="str">
-            <v>DB4299</v>
-          </cell>
-          <cell r="D48" t="str">
-            <v>BF463</v>
-          </cell>
-          <cell r="E48" t="str">
-            <v>FDR329253</v>
-          </cell>
-          <cell r="F48" t="str">
-            <v>BD-9617</v>
-          </cell>
-          <cell r="J48" t="str">
-            <v>BT-1300</v>
-          </cell>
-          <cell r="K48" t="str">
-            <v>AD5001</v>
-          </cell>
-          <cell r="L48" t="str">
-            <v>07050009</v>
-          </cell>
-          <cell r="M48" t="str">
-            <v>07050009</v>
-          </cell>
-          <cell r="N48" t="str">
-            <v>TFD-00617</v>
-          </cell>
-          <cell r="O48" t="str">
-            <v>BD200 4299</v>
-          </cell>
-          <cell r="Q48" t="str">
-            <v>BSG 90-225-001</v>
-          </cell>
-          <cell r="R48" t="str">
-            <v>94023800</v>
-          </cell>
-          <cell r="S48"/>
-          <cell r="T48" t="str">
-            <v>6Q0609617</v>
-          </cell>
-        </row>
-        <row r="49">
-          <cell r="A49">
-            <v>13544</v>
-          </cell>
-          <cell r="D49" t="str">
-            <v>BG4064</v>
-          </cell>
-          <cell r="K49" t="str">
-            <v>AD5016</v>
-          </cell>
-          <cell r="L49" t="str">
-            <v>07050023</v>
-          </cell>
-          <cell r="M49" t="str">
-            <v>07050023</v>
-          </cell>
-          <cell r="N49" t="str">
-            <v>TFD-00322</v>
-          </cell>
-          <cell r="O49" t="str">
-            <v>BDK200 4474</v>
-          </cell>
-          <cell r="Q49" t="str">
-            <v>BSG 30-225-019</v>
-          </cell>
-          <cell r="R49" t="str">
-            <v>94045600</v>
-          </cell>
-          <cell r="S49"/>
-          <cell r="T49" t="str">
-            <v>EY161126AA</v>
-          </cell>
-        </row>
-        <row r="50">
-          <cell r="A50">
-            <v>16561</v>
-          </cell>
-          <cell r="C50" t="str">
-            <v>DB4422</v>
-          </cell>
-          <cell r="K50" t="str">
-            <v>AD5013</v>
-          </cell>
-          <cell r="L50" t="str">
-            <v>07050008</v>
-          </cell>
-          <cell r="M50" t="str">
-            <v>07050008</v>
-          </cell>
-          <cell r="N50" t="str">
-            <v>TFD-00785</v>
-          </cell>
-          <cell r="O50" t="str">
-            <v>BDK200 4422</v>
-          </cell>
-          <cell r="P50" t="str">
-            <v>RAI-KD02010</v>
-          </cell>
-          <cell r="Q50" t="str">
-            <v>BSG 40-225-004</v>
-          </cell>
-          <cell r="R50" t="str">
-            <v>94035900</v>
-          </cell>
-          <cell r="S50"/>
-          <cell r="T50" t="str">
-            <v>584111G000</v>
-          </cell>
-        </row>
-        <row r="51">
-          <cell r="A51">
-            <v>34565</v>
-          </cell>
-          <cell r="B51" t="str">
-            <v>14.5815.10</v>
-          </cell>
-          <cell r="C51" t="str">
-            <v>DB4115, DB4256</v>
-          </cell>
-          <cell r="E51" t="str">
-            <v>FDR329088</v>
-          </cell>
-          <cell r="K51" t="str">
-            <v>AD5002</v>
-          </cell>
-          <cell r="L51" t="str">
-            <v>07050007</v>
-          </cell>
-          <cell r="M51" t="str">
-            <v>07050007</v>
-          </cell>
-          <cell r="O51" t="str">
-            <v>BDK300 34565</v>
-          </cell>
-          <cell r="P51" t="str">
-            <v>RAI-KC02032</v>
-          </cell>
-          <cell r="Q51" t="str">
-            <v>BSG 85-225-001</v>
-          </cell>
-          <cell r="T51" t="str">
-            <v>4243120250</v>
-          </cell>
-        </row>
-        <row r="52">
-          <cell r="A52">
-            <v>40569</v>
-          </cell>
-          <cell r="C52" t="str">
-            <v>DB4452</v>
-          </cell>
-          <cell r="D52" t="str">
-            <v>BF573</v>
-          </cell>
-          <cell r="F52" t="str">
-            <v>BD-3972</v>
-          </cell>
-          <cell r="K52" t="str">
-            <v>AD5042</v>
-          </cell>
-          <cell r="L52" t="str">
-            <v>07040274</v>
-          </cell>
-          <cell r="M52" t="str">
-            <v>07040274</v>
-          </cell>
-          <cell r="N52" t="str">
-            <v>TFD-00632</v>
-          </cell>
-          <cell r="P52" t="str">
-            <v>RAI-KD02012</v>
-          </cell>
-          <cell r="Q52" t="str">
-            <v>BSG 41-225-003</v>
-          </cell>
-          <cell r="R52" t="str">
-            <v>94039400</v>
-          </cell>
-          <cell r="S52"/>
-          <cell r="T52" t="str">
-            <v>8979480380</v>
-          </cell>
-        </row>
-        <row r="53">
-          <cell r="A53">
-            <v>36571</v>
-          </cell>
-          <cell r="B53" t="str">
-            <v>14.9384.10</v>
-          </cell>
-          <cell r="C53" t="str">
-            <v>DB4260</v>
-          </cell>
-          <cell r="D53" t="str">
-            <v>BF410</v>
-          </cell>
-          <cell r="F53" t="str">
-            <v>BD-9615</v>
-          </cell>
-          <cell r="K53" t="str">
-            <v>AD5023</v>
-          </cell>
-          <cell r="L53" t="str">
-            <v>07040210</v>
-          </cell>
-          <cell r="M53" t="str">
-            <v>07040210</v>
-          </cell>
-          <cell r="Q53" t="str">
-            <v>BSG 90-225-004</v>
-          </cell>
-          <cell r="R53" t="str">
-            <v>94022800</v>
-          </cell>
-          <cell r="S53"/>
-          <cell r="T53" t="str">
-            <v>6X0609617A</v>
-          </cell>
-        </row>
-        <row r="54">
-          <cell r="A54">
-            <v>30579</v>
-          </cell>
-          <cell r="B54" t="str">
-            <v>14.E312.60</v>
-          </cell>
-          <cell r="C54" t="str">
-            <v>DB4557MR</v>
-          </cell>
-          <cell r="K54" t="str">
-            <v>AD5005</v>
-          </cell>
-          <cell r="L54" t="str">
-            <v>07040371</v>
-          </cell>
-          <cell r="M54" t="str">
-            <v>07040371</v>
-          </cell>
-          <cell r="O54" t="str">
-            <v>BDK300 30579</v>
-          </cell>
-          <cell r="Q54" t="str">
-            <v>BSG 75-225-004</v>
-          </cell>
-          <cell r="T54" t="str">
-            <v>432007212R</v>
-          </cell>
-        </row>
-        <row r="55">
-          <cell r="A55">
-            <v>33591</v>
-          </cell>
-          <cell r="B55" t="str">
-            <v>14.A855.10</v>
-          </cell>
-          <cell r="C55" t="str">
-            <v>DB4360</v>
-          </cell>
-          <cell r="D55" t="str">
-            <v>BF503</v>
-          </cell>
-          <cell r="E55" t="str">
-            <v>FDR329801</v>
-          </cell>
-          <cell r="K55" t="str">
-            <v>AD5033</v>
-          </cell>
-          <cell r="L55" t="str">
-            <v>07050072</v>
-          </cell>
-          <cell r="M55" t="str">
-            <v>07050072</v>
-          </cell>
-          <cell r="O55" t="str">
-            <v>BDK300 33591</v>
-          </cell>
-          <cell r="Q55" t="str">
-            <v>BSG 65-225-006</v>
-          </cell>
-          <cell r="R55" t="str">
-            <v>94027200</v>
-          </cell>
-          <cell r="S55"/>
-          <cell r="T55" t="str">
-            <v>51901443</v>
-          </cell>
-        </row>
-        <row r="56">
-          <cell r="A56" t="str">
-            <v>30579B</v>
-          </cell>
-          <cell r="C56" t="str">
-            <v>DB4557MR</v>
-          </cell>
-          <cell r="K56" t="str">
-            <v>AD5004</v>
-          </cell>
-          <cell r="L56" t="str">
-            <v>07059371</v>
-          </cell>
-          <cell r="M56" t="str">
-            <v>07059371</v>
-          </cell>
-          <cell r="N56" t="str">
-            <v>TFD-00169</v>
-          </cell>
-          <cell r="O56" t="str">
-            <v>BD200 4557MR</v>
-          </cell>
-          <cell r="R56" t="str">
-            <v>94047400</v>
-          </cell>
-          <cell r="S56"/>
-          <cell r="T56" t="str">
-            <v>432007212R</v>
-          </cell>
-        </row>
-        <row r="57">
-          <cell r="A57">
-            <v>28593</v>
-          </cell>
-          <cell r="B57" t="str">
-            <v>14.7714.10</v>
-          </cell>
-          <cell r="C57" t="str">
-            <v>DB4211</v>
-          </cell>
-          <cell r="K57" t="str">
-            <v>AE1350</v>
-          </cell>
-          <cell r="L57" t="str">
-            <v>07040390</v>
-          </cell>
-          <cell r="M57" t="str">
-            <v>07040390</v>
-          </cell>
-          <cell r="T57" t="str">
-            <v>424640</v>
-          </cell>
-        </row>
-        <row r="58">
-          <cell r="A58">
-            <v>33740</v>
-          </cell>
-          <cell r="B58" t="str">
-            <v>14.7127.20</v>
-          </cell>
-          <cell r="C58" t="str">
-            <v>DB4210</v>
-          </cell>
-          <cell r="D58" t="str">
-            <v>BF379</v>
-          </cell>
-          <cell r="E58" t="str">
-            <v>FDR329006</v>
-          </cell>
-          <cell r="J58" t="str">
-            <v>BT-0560</v>
-          </cell>
-          <cell r="K58" t="str">
-            <v>AD5040</v>
-          </cell>
-          <cell r="L58" t="str">
-            <v>07050070</v>
-          </cell>
-          <cell r="M58" t="str">
-            <v>07050070</v>
-          </cell>
-          <cell r="O58" t="str">
-            <v>BDK300 33740</v>
-          </cell>
-          <cell r="Q58" t="str">
-            <v>BSG 25-225-002</v>
-          </cell>
-          <cell r="R58" t="str">
-            <v>94014000</v>
-          </cell>
-          <cell r="S58"/>
-          <cell r="T58" t="str">
-            <v>7769850</v>
-          </cell>
-        </row>
-        <row r="59">
-          <cell r="A59">
-            <v>26747</v>
-          </cell>
-          <cell r="K59" t="str">
-            <v>AD5049</v>
-          </cell>
-          <cell r="L59" t="str">
-            <v>07040492</v>
-          </cell>
-          <cell r="M59" t="str">
-            <v>07040492</v>
-          </cell>
-          <cell r="P59" t="str">
-            <v>RAI-KD02039</v>
-          </cell>
-          <cell r="Q59" t="str">
-            <v>BSG 63-225-001</v>
-          </cell>
-          <cell r="R59" t="str">
-            <v>94046500</v>
-          </cell>
-          <cell r="S59"/>
-          <cell r="T59" t="str">
-            <v>43206EB360</v>
-          </cell>
-        </row>
-        <row r="60">
-          <cell r="A60">
-            <v>15701</v>
-          </cell>
-          <cell r="C60" t="str">
-            <v>DB4020</v>
-          </cell>
-          <cell r="D60" t="str">
-            <v>BF208</v>
-          </cell>
-          <cell r="E60" t="str">
-            <v>FDR329061</v>
-          </cell>
-          <cell r="J60" t="str">
-            <v>BT-1350</v>
-          </cell>
-          <cell r="L60" t="str">
-            <v>07040468</v>
-          </cell>
-          <cell r="M60" t="str">
-            <v>07040468</v>
-          </cell>
-          <cell r="P60" t="str">
-            <v>RAI-KD02018</v>
-          </cell>
-          <cell r="Q60" t="str">
-            <v>BSG 35-225-002</v>
-          </cell>
-          <cell r="T60" t="str">
-            <v>42610SR3000</v>
-          </cell>
-        </row>
-        <row r="61">
-          <cell r="A61">
-            <v>15702</v>
-          </cell>
-          <cell r="E61" t="str">
-            <v>FDR329805</v>
-          </cell>
-          <cell r="K61" t="str">
-            <v>AD5052</v>
-          </cell>
-          <cell r="L61" t="str">
-            <v>07040380</v>
-          </cell>
-          <cell r="M61" t="str">
-            <v>07040380</v>
-          </cell>
-          <cell r="P61" t="str">
-            <v>RAI-KD02028</v>
-          </cell>
-          <cell r="Q61" t="str">
-            <v>BSG 35-225-003</v>
-          </cell>
-          <cell r="R61" t="str">
-            <v>94037100</v>
-          </cell>
-          <cell r="S61"/>
-          <cell r="T61" t="str">
-            <v>42610S5A000</v>
-          </cell>
-        </row>
-        <row r="62">
-          <cell r="A62">
-            <v>16703</v>
-          </cell>
-          <cell r="K62" t="str">
-            <v>AD5055</v>
-          </cell>
-          <cell r="L62" t="str">
-            <v>07040469</v>
-          </cell>
-          <cell r="M62" t="str">
-            <v>07040469</v>
-          </cell>
-          <cell r="P62" t="str">
-            <v>RAI-KD02036</v>
-          </cell>
-          <cell r="T62" t="str">
-            <v>583294A200</v>
-          </cell>
-        </row>
-        <row r="63">
-          <cell r="A63">
-            <v>16704</v>
-          </cell>
-          <cell r="K63" t="str">
-            <v>AD5047</v>
-          </cell>
-          <cell r="L63" t="str">
-            <v>07040470</v>
-          </cell>
-          <cell r="M63" t="str">
-            <v>07040470</v>
-          </cell>
-          <cell r="P63" t="str">
-            <v>RAI-KD02029</v>
-          </cell>
-          <cell r="Q63" t="str">
-            <v>BSG 40-225-013</v>
-          </cell>
-          <cell r="T63" t="str">
-            <v>5276147010</v>
-          </cell>
-        </row>
-        <row r="64">
-          <cell r="A64">
-            <v>16705</v>
-          </cell>
-          <cell r="C64" t="str">
-            <v>DB4267</v>
-          </cell>
-          <cell r="D64" t="str">
-            <v>BF435</v>
-          </cell>
-          <cell r="F64" t="str">
-            <v>FDR329319</v>
-          </cell>
-          <cell r="J64" t="str">
-            <v>BT-1530</v>
-          </cell>
-          <cell r="K64" t="str">
-            <v>AD5046</v>
-          </cell>
-          <cell r="L64" t="str">
-            <v>07040471</v>
-          </cell>
-          <cell r="M64" t="str">
-            <v>07040471</v>
-          </cell>
-          <cell r="P64" t="str">
-            <v>RAI-KD02016</v>
-          </cell>
-          <cell r="Q64" t="str">
-            <v>BSG 40-225-014</v>
-          </cell>
-          <cell r="T64" t="str">
-            <v>5841122100</v>
-          </cell>
-        </row>
-        <row r="65">
-          <cell r="A65">
-            <v>16706</v>
-          </cell>
-          <cell r="C65" t="str">
-            <v>DB4283</v>
-          </cell>
-          <cell r="D65" t="str">
-            <v>BF435</v>
-          </cell>
-          <cell r="E65" t="str">
-            <v>FDR329321</v>
-          </cell>
-          <cell r="J65" t="str">
-            <v>BT-1850</v>
-          </cell>
-          <cell r="L65" t="str">
-            <v>07040472</v>
-          </cell>
-          <cell r="M65" t="str">
-            <v>07040472</v>
-          </cell>
-          <cell r="O65" t="str">
-            <v>BD200 4283</v>
-          </cell>
-          <cell r="P65" t="str">
-            <v>RAI-KD02015</v>
-          </cell>
-          <cell r="Q65" t="str">
-            <v>BSG 40-225-008</v>
-          </cell>
-          <cell r="T65" t="str">
-            <v>5841122000</v>
-          </cell>
-        </row>
-        <row r="66">
-          <cell r="A66">
-            <v>16707</v>
-          </cell>
-          <cell r="B66" t="str">
-            <v>14.C013.10</v>
-          </cell>
-          <cell r="C66" t="str">
-            <v>DB4402</v>
-          </cell>
-          <cell r="D66" t="str">
-            <v>BF519</v>
-          </cell>
-          <cell r="F66" t="str">
-            <v>BD-5200</v>
-          </cell>
-          <cell r="K66" t="str">
-            <v>AD5045</v>
-          </cell>
-          <cell r="L66" t="str">
-            <v>07040473</v>
-          </cell>
-          <cell r="M66" t="str">
-            <v>07040473</v>
-          </cell>
-          <cell r="P66" t="str">
-            <v>RAI-KD02020</v>
-          </cell>
-          <cell r="T66" t="str">
-            <v>5841125010</v>
-          </cell>
-        </row>
-        <row r="67">
-          <cell r="A67">
-            <v>16708</v>
-          </cell>
-          <cell r="C67" t="str">
-            <v>DB4416</v>
-          </cell>
-          <cell r="E67" t="str">
-            <v>FDR329319</v>
-          </cell>
-          <cell r="K67" t="str">
-            <v>AD5054</v>
-          </cell>
-          <cell r="L67" t="str">
-            <v>07040474</v>
-          </cell>
-          <cell r="M67" t="str">
-            <v>07040474</v>
-          </cell>
-          <cell r="P67" t="str">
-            <v>RAI-KD02024</v>
-          </cell>
-          <cell r="Q67" t="str">
-            <v>BSG 40-225-010</v>
-          </cell>
-          <cell r="T67" t="str">
-            <v>5841125201</v>
-          </cell>
-        </row>
-        <row r="68">
-          <cell r="A68">
-            <v>16709</v>
-          </cell>
-          <cell r="C68" t="str">
-            <v>DB4430</v>
-          </cell>
-          <cell r="D68" t="str">
-            <v>BF551</v>
-          </cell>
-          <cell r="K68" t="str">
-            <v>AD5044</v>
-          </cell>
-          <cell r="L68" t="str">
-            <v>07040475</v>
-          </cell>
-          <cell r="M68" t="str">
-            <v>07040475</v>
-          </cell>
-          <cell r="P68" t="str">
-            <v>RAI-KD02014</v>
-          </cell>
-          <cell r="Q68" t="str">
-            <v>BSG 40-225-011</v>
-          </cell>
-          <cell r="T68" t="str">
-            <v>584111C000</v>
-          </cell>
-        </row>
-        <row r="69">
-          <cell r="A69">
-            <v>16710</v>
-          </cell>
-          <cell r="C69" t="str">
-            <v>DB4401</v>
-          </cell>
-          <cell r="D69" t="str">
-            <v>BF517</v>
-          </cell>
-          <cell r="E69" t="str">
-            <v>FDR329755</v>
-          </cell>
-          <cell r="J69" t="str">
-            <v>BT-2130</v>
-          </cell>
-          <cell r="K69" t="str">
-            <v>AD5058</v>
-          </cell>
-          <cell r="L69" t="str">
-            <v>07040386</v>
-          </cell>
-          <cell r="M69" t="str">
-            <v>07040386</v>
-          </cell>
-          <cell r="O69" t="str">
-            <v>BD200 4401</v>
-          </cell>
-          <cell r="P69" t="str">
-            <v>RAI-KD02022</v>
-          </cell>
-          <cell r="Q69" t="str">
-            <v>BSG 40-225-009</v>
-          </cell>
-          <cell r="R69" t="str">
-            <v>94033300</v>
-          </cell>
-          <cell r="S69"/>
-          <cell r="T69" t="str">
-            <v>584111C300</v>
-          </cell>
-        </row>
-        <row r="70">
-          <cell r="A70">
-            <v>18711</v>
-          </cell>
-          <cell r="B70" t="str">
-            <v>14.9394.10</v>
-          </cell>
-          <cell r="C70" t="str">
-            <v>DB4322</v>
-          </cell>
-          <cell r="E70" t="str">
-            <v>FDR329345</v>
-          </cell>
-          <cell r="F70" t="str">
-            <v>BD-0006</v>
-          </cell>
-          <cell r="K70" t="str">
-            <v>AD5074</v>
-          </cell>
-          <cell r="L70" t="str">
-            <v>07040480</v>
-          </cell>
-          <cell r="M70" t="str">
-            <v>07040480</v>
-          </cell>
-          <cell r="P70" t="str">
-            <v>RAI-KD02035</v>
-          </cell>
-          <cell r="Q70" t="str">
-            <v>BSG 55-225-003</v>
-          </cell>
-          <cell r="T70" t="str">
-            <v>0S08326251B</v>
-          </cell>
-        </row>
-        <row r="71">
-          <cell r="A71">
-            <v>22712</v>
-          </cell>
-          <cell r="B71" t="str">
-            <v>14.A700.10</v>
-          </cell>
-          <cell r="C71" t="str">
-            <v>DB4345</v>
-          </cell>
-          <cell r="E71" t="str">
-            <v>FDR329322</v>
-          </cell>
-          <cell r="K71" t="str">
-            <v>AD5075</v>
-          </cell>
-          <cell r="L71" t="str">
-            <v>07040483</v>
-          </cell>
-          <cell r="M71" t="str">
-            <v>07040483</v>
-          </cell>
-          <cell r="P71" t="str">
-            <v>RAI-KC02037</v>
-          </cell>
-          <cell r="Q71" t="str">
-            <v>BSG 55-225-001</v>
-          </cell>
-          <cell r="T71" t="str">
-            <v>B45526251</v>
-          </cell>
-        </row>
-        <row r="72">
-          <cell r="A72">
-            <v>22713</v>
-          </cell>
-          <cell r="B72" t="str">
-            <v>14.D631.10</v>
-          </cell>
-          <cell r="C72" t="str">
-            <v>DB4279</v>
-          </cell>
-          <cell r="D72" t="str">
-            <v>BF456</v>
-          </cell>
-          <cell r="E72" t="str">
-            <v>FDR329322</v>
-          </cell>
-          <cell r="J72" t="str">
-            <v>BT-2250</v>
-          </cell>
-          <cell r="L72" t="str">
-            <v>07040484</v>
-          </cell>
-          <cell r="M72" t="str">
-            <v>07040484</v>
-          </cell>
-          <cell r="P72" t="str">
-            <v>RAI-KD02017</v>
-          </cell>
-          <cell r="Q72" t="str">
-            <v>BSG 55-225-004</v>
-          </cell>
-          <cell r="T72" t="str">
-            <v>B59626251</v>
-          </cell>
-        </row>
-        <row r="73">
-          <cell r="A73">
-            <v>22714</v>
-          </cell>
-          <cell r="L73" t="str">
-            <v>07040485</v>
-          </cell>
-          <cell r="M73" t="str">
-            <v>07040485</v>
-          </cell>
-          <cell r="P73" t="str">
-            <v>RAI-KD02030</v>
-          </cell>
-          <cell r="Q73" t="str">
-            <v>BSG 55-225-002</v>
-          </cell>
-          <cell r="T73" t="str">
-            <v>GJ2126251</v>
-          </cell>
-        </row>
-        <row r="74">
-          <cell r="A74">
-            <v>26715</v>
-          </cell>
-          <cell r="C74" t="str">
-            <v>DB4249</v>
-          </cell>
-          <cell r="D74" t="str">
-            <v>BF461</v>
-          </cell>
-          <cell r="E74" t="str">
-            <v>FDR329306</v>
-          </cell>
-          <cell r="K74" t="str">
-            <v>AD5051</v>
-          </cell>
-          <cell r="L74" t="str">
-            <v>07040491</v>
-          </cell>
-          <cell r="M74" t="str">
-            <v>07040491</v>
-          </cell>
-          <cell r="P74" t="str">
-            <v>RAI-KD02040</v>
-          </cell>
-          <cell r="Q74" t="str">
-            <v>BSG 63-225-002</v>
-          </cell>
-          <cell r="R74" t="str">
-            <v>94036700</v>
-          </cell>
-          <cell r="S74"/>
-          <cell r="T74" t="str">
-            <v>432062S600</v>
-          </cell>
-        </row>
-        <row r="75">
-          <cell r="A75">
-            <v>32716</v>
-          </cell>
-          <cell r="C75" t="str">
-            <v>DB4233</v>
-          </cell>
-          <cell r="D75" t="str">
-            <v>BF447</v>
-          </cell>
-          <cell r="E75" t="str">
-            <v>FDR329310</v>
-          </cell>
-          <cell r="L75" t="str">
-            <v>07040391</v>
-          </cell>
-          <cell r="M75" t="str">
-            <v>07040391</v>
-          </cell>
-          <cell r="P75" t="str">
-            <v>RAI-KD02031</v>
-          </cell>
-          <cell r="Q75" t="str">
-            <v>BSG 83-225-002</v>
-          </cell>
-          <cell r="T75" t="str">
-            <v>4351177E00</v>
-          </cell>
-        </row>
-        <row r="76">
-          <cell r="A76">
-            <v>34717</v>
-          </cell>
-          <cell r="B76" t="str">
-            <v>14.4785.10</v>
-          </cell>
-          <cell r="J76" t="str">
-            <v>BT-1730</v>
-          </cell>
-          <cell r="K76" t="str">
-            <v>AD5077</v>
-          </cell>
-          <cell r="L76" t="str">
-            <v>07040393</v>
-          </cell>
-          <cell r="M76" t="str">
-            <v>07040393</v>
-          </cell>
-          <cell r="P76" t="str">
-            <v>RAI-KD02027</v>
-          </cell>
-          <cell r="Q76" t="str">
-            <v>BSG 85-225-005</v>
-          </cell>
-          <cell r="T76" t="str">
-            <v>4243135151</v>
-          </cell>
-        </row>
-        <row r="77">
-          <cell r="A77">
-            <v>34718</v>
-          </cell>
-          <cell r="B77" t="str">
-            <v>14.D636.10</v>
-          </cell>
-          <cell r="E77" t="str">
-            <v>FDR329804</v>
-          </cell>
-          <cell r="K77" t="str">
-            <v>AD5026</v>
-          </cell>
-          <cell r="L77" t="str">
-            <v>07040496</v>
-          </cell>
-          <cell r="M77" t="str">
-            <v>07040496</v>
-          </cell>
-          <cell r="P77" t="str">
-            <v>RAI-KD02033</v>
-          </cell>
-          <cell r="Q77" t="str">
-            <v>BSG 85-225-006</v>
-          </cell>
-          <cell r="R77" t="str">
-            <v>94038600</v>
-          </cell>
-          <cell r="S77"/>
-          <cell r="T77" t="str">
-            <v>424310K080</v>
-          </cell>
-        </row>
-        <row r="78">
-          <cell r="A78">
-            <v>34719</v>
-          </cell>
-          <cell r="C78" t="str">
-            <v>DB7036</v>
-          </cell>
-          <cell r="E78" t="str">
-            <v>FDR329795</v>
-          </cell>
-          <cell r="J78" t="str">
-            <v>BT-2030</v>
-          </cell>
-          <cell r="K78" t="str">
-            <v>AD5025</v>
-          </cell>
-          <cell r="L78" t="str">
-            <v>07040497</v>
-          </cell>
-          <cell r="M78" t="str">
-            <v>07040497</v>
-          </cell>
-          <cell r="P78" t="str">
-            <v>RAI-KD02038</v>
-          </cell>
-          <cell r="Q78" t="str">
-            <v>BSG 85-225-007</v>
-          </cell>
-          <cell r="R78" t="str">
-            <v>94038800</v>
-          </cell>
-          <cell r="S78"/>
-          <cell r="T78" t="str">
-            <v>424310K120</v>
-          </cell>
-        </row>
-        <row r="79">
-          <cell r="A79">
-            <v>34720</v>
-          </cell>
-          <cell r="B79" t="str">
-            <v>14.9378.10</v>
-          </cell>
-          <cell r="K79" t="str">
-            <v>AD5061</v>
-          </cell>
-          <cell r="L79" t="str">
-            <v>07040394</v>
-          </cell>
-          <cell r="M79" t="str">
-            <v>07040394</v>
-          </cell>
-          <cell r="P79" t="str">
-            <v>RAI-KD02023</v>
-          </cell>
-          <cell r="Q79" t="str">
-            <v>BSG 85-225-002</v>
-          </cell>
-          <cell r="R79" t="str">
-            <v>94029300</v>
-          </cell>
-          <cell r="S79"/>
-          <cell r="T79" t="str">
-            <v>4243152020</v>
-          </cell>
-        </row>
-        <row r="80">
-          <cell r="A80">
-            <v>34722</v>
-          </cell>
-          <cell r="B80" t="str">
-            <v>14.9379.10</v>
-          </cell>
-          <cell r="C80" t="str">
-            <v>DB4257</v>
-          </cell>
-          <cell r="D80" t="str">
-            <v>BF405</v>
-          </cell>
-          <cell r="E80" t="str">
-            <v>FDR329350</v>
-          </cell>
-          <cell r="J80" t="str">
-            <v>BT-2170</v>
-          </cell>
-          <cell r="K80" t="str">
-            <v>AD5060</v>
-          </cell>
-          <cell r="L80" t="str">
-            <v>07040498</v>
-          </cell>
-          <cell r="M80" t="str">
-            <v>07040498</v>
-          </cell>
-          <cell r="O80" t="str">
-            <v>BD200 4257</v>
-          </cell>
-          <cell r="P80" t="str">
-            <v>RAI-KD02026</v>
-          </cell>
-          <cell r="Q80" t="str">
-            <v>BSG 85-225-004</v>
-          </cell>
-          <cell r="T80" t="str">
-            <v>4243105020</v>
-          </cell>
-        </row>
-        <row r="81">
-          <cell r="A81">
-            <v>15723</v>
-          </cell>
-          <cell r="B81" t="str">
-            <v>14.7739.10</v>
-          </cell>
-          <cell r="C81" t="str">
-            <v>DB4223</v>
-          </cell>
-          <cell r="D81" t="str">
-            <v>BF419</v>
-          </cell>
-          <cell r="E81" t="str">
-            <v>FDR329063</v>
-          </cell>
-          <cell r="J81" t="str">
-            <v>BT-1870</v>
-          </cell>
-          <cell r="K81" t="str">
-            <v>AD5073</v>
-          </cell>
-          <cell r="L81" t="str">
-            <v>07040381</v>
-          </cell>
-          <cell r="M81" t="str">
-            <v>07040381</v>
-          </cell>
-          <cell r="P81" t="str">
-            <v>RAI-KD02025</v>
-          </cell>
-          <cell r="Q81" t="str">
-            <v>BSG 35-225-001</v>
-          </cell>
-          <cell r="R81" t="str">
-            <v>94023000</v>
-          </cell>
-          <cell r="S81"/>
-          <cell r="T81" t="str">
-            <v>42610S70000</v>
-          </cell>
-        </row>
-        <row r="82">
-          <cell r="A82">
-            <v>25728</v>
-          </cell>
-          <cell r="C82" t="str">
-            <v>DB4408</v>
-          </cell>
-          <cell r="D82" t="str">
-            <v>BF532</v>
-          </cell>
-          <cell r="F82" t="str">
-            <v>BD-7044</v>
-          </cell>
-          <cell r="J82" t="str">
-            <v>BT-1600</v>
-          </cell>
-          <cell r="K82" t="str">
-            <v>AD5039</v>
-          </cell>
-          <cell r="L82" t="str">
-            <v>07040487</v>
-          </cell>
-          <cell r="M82" t="str">
-            <v>07040487</v>
-          </cell>
-          <cell r="O82" t="str">
-            <v>BD200 4408</v>
-          </cell>
-          <cell r="P82" t="str">
-            <v>RAI-KD02037</v>
-          </cell>
-          <cell r="Q82" t="str">
-            <v>BSG 62-225-004</v>
-          </cell>
-          <cell r="T82" t="str">
-            <v>MB895470</v>
-          </cell>
-        </row>
-        <row r="83">
-          <cell r="A83">
-            <v>32734</v>
-          </cell>
-          <cell r="B83" t="str">
-            <v>14.9388.10</v>
-          </cell>
-          <cell r="C83" t="str">
-            <v>DB4269</v>
-          </cell>
-          <cell r="D83" t="str">
-            <v>BF449</v>
-          </cell>
-          <cell r="E83" t="str">
-            <v>FDR329288</v>
-          </cell>
-          <cell r="F83" t="str">
-            <v>BD-4810</v>
-          </cell>
-          <cell r="J83" t="str">
-            <v>BT-1490</v>
-          </cell>
-          <cell r="K83" t="str">
-            <v>AD5053</v>
-          </cell>
-          <cell r="L83" t="str">
-            <v>07040493</v>
-          </cell>
-          <cell r="M83" t="str">
-            <v>07040493</v>
-          </cell>
-          <cell r="P83" t="str">
-            <v>RAI-KD02021</v>
-          </cell>
-          <cell r="Q83" t="str">
-            <v>BSG 83-225-001</v>
-          </cell>
-          <cell r="T83" t="str">
-            <v>4351160G00</v>
-          </cell>
-        </row>
-        <row r="84">
-          <cell r="A84">
-            <v>32735</v>
-          </cell>
-          <cell r="C84" t="str">
-            <v>DB4362</v>
-          </cell>
-          <cell r="D84" t="str">
-            <v>BF506</v>
-          </cell>
-          <cell r="E84" t="str">
-            <v>FDR329265</v>
-          </cell>
-          <cell r="F84" t="str">
-            <v>BD-4701</v>
-          </cell>
-          <cell r="J84" t="str">
-            <v>BT-2100</v>
-          </cell>
-          <cell r="K84" t="str">
-            <v>AD5056</v>
-          </cell>
-          <cell r="L84" t="str">
-            <v>07040494</v>
-          </cell>
-          <cell r="M84" t="str">
-            <v>07040494</v>
-          </cell>
-          <cell r="O84" t="str">
-            <v>BD200 4362</v>
-          </cell>
-          <cell r="R84" t="str">
-            <v>94026500</v>
-          </cell>
-          <cell r="S84"/>
-          <cell r="T84" t="str">
-            <v>424748</v>
-          </cell>
-        </row>
-        <row r="85">
-          <cell r="A85">
-            <v>34739</v>
-          </cell>
-          <cell r="C85" t="str">
-            <v>DB4339</v>
-          </cell>
-          <cell r="D85" t="str">
-            <v>BF530</v>
-          </cell>
-          <cell r="K85" t="str">
-            <v>AD5062</v>
-          </cell>
-          <cell r="L85" t="str">
-            <v>07040395</v>
-          </cell>
-          <cell r="M85" t="str">
-            <v>07040395</v>
-          </cell>
-          <cell r="P85" t="str">
-            <v>RAI-KD02019</v>
-          </cell>
-          <cell r="Q85" t="str">
-            <v>BSG 85-225-003</v>
-          </cell>
-          <cell r="R85" t="str">
-            <v>94034600</v>
-          </cell>
-          <cell r="S85"/>
-          <cell r="T85" t="str">
-            <v>424310D010</v>
-          </cell>
-        </row>
-        <row r="86">
-          <cell r="A86">
-            <v>37737</v>
-          </cell>
-          <cell r="M86"/>
-          <cell r="T86"/>
-        </row>
-        <row r="87">
-          <cell r="A87">
-            <v>27762</v>
-          </cell>
-          <cell r="C87" t="str">
-            <v>DB4302</v>
-          </cell>
-          <cell r="D87" t="str">
-            <v>BF472</v>
-          </cell>
-          <cell r="E87" t="str">
-            <v>FDR329259</v>
-          </cell>
-          <cell r="F87" t="str">
-            <v>BD-8001</v>
-          </cell>
-          <cell r="J87" t="str">
-            <v>BT-2260</v>
-          </cell>
-          <cell r="K87" t="str">
-            <v>AD5034</v>
-          </cell>
-          <cell r="L87" t="str">
-            <v>07050063</v>
-          </cell>
-          <cell r="M87" t="str">
-            <v>07050063</v>
-          </cell>
-          <cell r="O87" t="str">
-            <v>BD200 4302</v>
-          </cell>
-          <cell r="Q87" t="str">
-            <v>BSG 65-225-005</v>
-          </cell>
-          <cell r="R87" t="str">
-            <v>94024200</v>
-          </cell>
-          <cell r="S87"/>
-          <cell r="T87" t="str">
-            <v>418001</v>
-          </cell>
-        </row>
-        <row r="88">
-          <cell r="A88">
-            <v>30777</v>
-          </cell>
-          <cell r="B88" t="str">
-            <v>14.5591.10</v>
-          </cell>
-          <cell r="C88" t="str">
-            <v>DB4072</v>
-          </cell>
-          <cell r="D88" t="str">
-            <v>BF273</v>
-          </cell>
-          <cell r="E88" t="str">
-            <v>FDR329219</v>
-          </cell>
-          <cell r="F88" t="str">
-            <v>BD-0511</v>
-          </cell>
-          <cell r="L88" t="str">
-            <v>07050094</v>
-          </cell>
-          <cell r="M88" t="str">
-            <v>07050094</v>
-          </cell>
-          <cell r="R88" t="str">
-            <v>94013700</v>
-          </cell>
-          <cell r="S88"/>
-          <cell r="T88" t="str">
-            <v>7700710511</v>
-          </cell>
-        </row>
-        <row r="89">
-          <cell r="A89">
-            <v>33783</v>
-          </cell>
-          <cell r="B89" t="str">
-            <v>14.7260.10</v>
-          </cell>
-          <cell r="C89" t="str">
-            <v>DB4295</v>
-          </cell>
-          <cell r="L89" t="str">
-            <v>07050097</v>
-          </cell>
-          <cell r="M89" t="str">
-            <v>07050097</v>
-          </cell>
-          <cell r="R89" t="str">
-            <v>94020000</v>
-          </cell>
-          <cell r="S89"/>
-          <cell r="T89" t="str">
-            <v>5923606</v>
-          </cell>
-        </row>
-        <row r="90">
-          <cell r="A90">
-            <v>16789</v>
-          </cell>
-          <cell r="C90" t="str">
-            <v>DB4225</v>
-          </cell>
-          <cell r="D90" t="str">
-            <v>BF433</v>
-          </cell>
-          <cell r="E90" t="str">
-            <v>FDR329274</v>
-          </cell>
-          <cell r="K90" t="str">
-            <v>AD1122</v>
-          </cell>
-          <cell r="L90" t="str">
-            <v>07050085</v>
-          </cell>
-          <cell r="M90" t="str">
-            <v>07050085</v>
-          </cell>
-          <cell r="Q90" t="str">
-            <v>BSG 40-225-015</v>
-          </cell>
-          <cell r="R90" t="str">
-            <v>94034900</v>
-          </cell>
-          <cell r="S90"/>
-          <cell r="T90" t="str">
-            <v>5841117200</v>
-          </cell>
-        </row>
-        <row r="91">
-          <cell r="A91">
-            <v>16790</v>
-          </cell>
-          <cell r="F91" t="str">
-            <v>BD-5188</v>
-          </cell>
-          <cell r="K91" t="str">
-            <v>AD1123</v>
-          </cell>
-          <cell r="L91" t="str">
-            <v>07050086</v>
-          </cell>
-          <cell r="M91" t="str">
-            <v>07050086</v>
-          </cell>
-          <cell r="Q91" t="str">
-            <v>BSG 40-225-012</v>
-          </cell>
-          <cell r="R91" t="str">
-            <v>94046700</v>
-          </cell>
-          <cell r="S91"/>
-          <cell r="T91" t="str">
-            <v>584111R000</v>
-          </cell>
-        </row>
-        <row r="92">
-          <cell r="A92">
-            <v>42804</v>
-          </cell>
-          <cell r="L92" t="str">
-            <v>07050066</v>
-          </cell>
-          <cell r="M92" t="str">
-            <v>07050066</v>
-          </cell>
-          <cell r="Q92" t="str">
-            <v>BSG 80-225-002</v>
-          </cell>
-          <cell r="R92" t="str">
-            <v>94046000</v>
-          </cell>
-          <cell r="S92"/>
-          <cell r="T92" t="str">
-            <v>6R0609617B</v>
-          </cell>
-        </row>
-        <row r="93">
-          <cell r="A93">
-            <v>36815</v>
-          </cell>
-          <cell r="D93" t="str">
-            <v>BF558</v>
-          </cell>
-          <cell r="F93" t="str">
-            <v>BD-6383</v>
-          </cell>
-          <cell r="J93" t="str">
-            <v>BT-2310</v>
-          </cell>
-          <cell r="K93" t="str">
-            <v>AD5078</v>
-          </cell>
-          <cell r="L93" t="str">
-            <v>07050069</v>
-          </cell>
-          <cell r="M93" t="str">
-            <v>07050069</v>
-          </cell>
-          <cell r="Q93" t="str">
-            <v>BSG 90-225-005</v>
-          </cell>
-          <cell r="R93" t="str">
-            <v>94043900</v>
-          </cell>
-          <cell r="S93"/>
-          <cell r="T93" t="str">
-            <v>2H0609617</v>
-          </cell>
-        </row>
-        <row r="94">
-          <cell r="A94">
-            <v>30819</v>
-          </cell>
-          <cell r="B94" t="str">
-            <v>14.5493.10</v>
-          </cell>
-          <cell r="L94" t="str">
-            <v>07050095</v>
-          </cell>
-          <cell r="M94" t="str">
-            <v>07050095</v>
-          </cell>
-          <cell r="Q94" t="str">
-            <v>BSG 75-225-005</v>
-          </cell>
-          <cell r="T94" t="str">
-            <v>7700685473</v>
-          </cell>
-        </row>
-        <row r="95">
-          <cell r="A95">
-            <v>31820</v>
-          </cell>
-          <cell r="B95" t="str">
-            <v>14.9386.10</v>
-          </cell>
-          <cell r="K95" t="str">
-            <v>AD5076</v>
-          </cell>
-          <cell r="L95" t="str">
-            <v>07050067</v>
-          </cell>
-          <cell r="M95" t="str">
-            <v>07050067</v>
-          </cell>
-          <cell r="Q95" t="str">
-            <v>BSG 80-225-001</v>
-          </cell>
-          <cell r="R95" t="str">
-            <v>94024300</v>
-          </cell>
-          <cell r="S95"/>
-          <cell r="T95" t="str">
-            <v>1J0609617B</v>
-          </cell>
-        </row>
-        <row r="96">
-          <cell r="A96">
-            <v>33824</v>
-          </cell>
-          <cell r="B96" t="str">
-            <v>14.6755.10</v>
-          </cell>
-          <cell r="F96" t="str">
-            <v>BD-9325</v>
-          </cell>
-          <cell r="K96" t="str">
-            <v>AD5079</v>
-          </cell>
-          <cell r="L96" t="str">
-            <v>07050073</v>
-          </cell>
-          <cell r="M96" t="str">
-            <v>07050073</v>
-          </cell>
-          <cell r="R96" t="str">
-            <v>94014800</v>
-          </cell>
-          <cell r="S96"/>
-          <cell r="T96" t="str">
-            <v>46819776</v>
-          </cell>
-        </row>
-        <row r="97">
-          <cell r="A97">
-            <v>29825</v>
-          </cell>
-          <cell r="B97" t="str">
-            <v>14.7093.10</v>
-          </cell>
-          <cell r="L97" t="str">
-            <v>07050088</v>
-          </cell>
-          <cell r="M97" t="str">
-            <v>07050088</v>
-          </cell>
-          <cell r="R97" t="str">
-            <v>94014200</v>
-          </cell>
-          <cell r="S97"/>
-          <cell r="T97" t="str">
-            <v>424735</v>
-          </cell>
-        </row>
-        <row r="98">
-          <cell r="A98">
-            <v>29826</v>
-          </cell>
-          <cell r="K98" t="str">
-            <v>AD5113</v>
-          </cell>
-          <cell r="L98" t="str">
-            <v>07050089</v>
-          </cell>
-          <cell r="M98" t="str">
-            <v>07050089</v>
-          </cell>
-          <cell r="R98" t="str">
-            <v>94028200</v>
-          </cell>
-          <cell r="S98"/>
-          <cell r="T98" t="str">
-            <v>424741</v>
-          </cell>
-        </row>
-        <row r="99">
-          <cell r="A99">
-            <v>33827</v>
-          </cell>
-          <cell r="B99" t="str">
-            <v>14.3157.10</v>
-          </cell>
-          <cell r="K99" t="str">
-            <v>AD5115</v>
-          </cell>
-          <cell r="L99" t="str">
-            <v>07050098</v>
-          </cell>
-          <cell r="M99" t="str">
-            <v>07050098</v>
-          </cell>
-          <cell r="O99" t="str">
-            <v>BDK300 33827</v>
-          </cell>
-          <cell r="T99" t="str">
-            <v>85015914</v>
-          </cell>
-        </row>
-        <row r="100">
-          <cell r="A100">
-            <v>18911</v>
-          </cell>
-          <cell r="K100" t="str">
-            <v>AD1109</v>
-          </cell>
-          <cell r="L100" t="str">
-            <v>07050057</v>
-          </cell>
-          <cell r="M100" t="str">
-            <v>07050057</v>
-          </cell>
-          <cell r="P100" t="str">
-            <v>RAI-KD02041</v>
-          </cell>
-          <cell r="T100" t="str">
-            <v>584114E000</v>
-          </cell>
-        </row>
-        <row r="101">
-          <cell r="A101">
-            <v>33976</v>
-          </cell>
-          <cell r="B101" t="str">
-            <v>14.3161.10</v>
-          </cell>
-          <cell r="K101" t="str">
-            <v>AD5080</v>
-          </cell>
-          <cell r="L101" t="str">
-            <v>07050092</v>
-          </cell>
-          <cell r="M101" t="str">
-            <v>07050092</v>
-          </cell>
-          <cell r="R101" t="str">
-            <v>94010200</v>
-          </cell>
-          <cell r="S101"/>
-          <cell r="T101" t="str">
-            <v>4449694</v>
-          </cell>
-        </row>
-        <row r="102">
-          <cell r="A102">
-            <v>33987</v>
-          </cell>
-          <cell r="B102" t="str">
-            <v>14.3157.20</v>
-          </cell>
-          <cell r="T102" t="str">
-            <v>5923924</v>
-          </cell>
-        </row>
-        <row r="103">
-          <cell r="A103">
-            <v>28988</v>
-          </cell>
-          <cell r="D103" t="str">
-            <v>BFR484</v>
-          </cell>
-          <cell r="E103" t="str">
-            <v>FDR329716</v>
-          </cell>
-          <cell r="R103" t="str">
-            <v>94026600</v>
-          </cell>
-          <cell r="S103"/>
-          <cell r="T103" t="str">
-            <v>424746</v>
-          </cell>
-        </row>
-        <row r="104">
-          <cell r="A104" t="str">
-            <v>45387H</v>
-          </cell>
-          <cell r="M104"/>
-          <cell r="T104" t="str">
-            <v>3757089</v>
-          </cell>
-        </row>
-        <row r="105">
-          <cell r="A105">
-            <v>33992</v>
-          </cell>
-          <cell r="C105" t="str">
-            <v>DB4563</v>
-          </cell>
-          <cell r="D105" t="str">
-            <v>BF379</v>
-          </cell>
-          <cell r="E105" t="str">
-            <v>FDR329006</v>
-          </cell>
-          <cell r="K105" t="str">
-            <v>AD5090</v>
-          </cell>
-          <cell r="L105" t="str">
-            <v>07050071</v>
-          </cell>
-          <cell r="M105" t="str">
-            <v>07050071</v>
-          </cell>
-          <cell r="O105" t="str">
-            <v>BDK300 33392</v>
-          </cell>
-          <cell r="T105" t="str">
-            <v>51860868</v>
-          </cell>
-        </row>
-        <row r="106">
-          <cell r="A106">
-            <v>30997</v>
-          </cell>
-          <cell r="K106" t="str">
-            <v>AD1132</v>
-          </cell>
-          <cell r="L106" t="str">
-            <v>07050096</v>
-          </cell>
-          <cell r="M106" t="str">
-            <v>07050096</v>
-          </cell>
-          <cell r="T106" t="str">
-            <v>432004334R</v>
-          </cell>
-        </row>
-        <row r="107">
-          <cell r="A107">
-            <v>161065</v>
-          </cell>
-          <cell r="F107" t="str">
-            <v>BD-5204</v>
-          </cell>
-          <cell r="L107" t="str">
-            <v>07050084</v>
-          </cell>
-          <cell r="M107"/>
-          <cell r="T107" t="str">
-            <v>584111S100</v>
-          </cell>
-        </row>
-        <row r="108">
-          <cell r="A108">
-            <v>291066</v>
-          </cell>
-          <cell r="I108" t="str">
-            <v>251919</v>
-          </cell>
-          <cell r="K108" t="str">
-            <v>AD5114</v>
-          </cell>
-          <cell r="L108" t="str">
-            <v>07050090</v>
-          </cell>
-          <cell r="M108" t="str">
-            <v>07050090</v>
-          </cell>
-          <cell r="O108" t="str">
-            <v>BDK300 29166</v>
-          </cell>
-          <cell r="T108" t="str">
-            <v>424759</v>
-          </cell>
-        </row>
-        <row r="109">
-          <cell r="A109">
-            <v>63999</v>
-          </cell>
-          <cell r="T109" t="str">
-            <v>3302350207001</v>
-          </cell>
-        </row>
-        <row r="110">
-          <cell r="A110">
-            <v>251070</v>
-          </cell>
-          <cell r="T110" t="str">
-            <v>MC862229</v>
-          </cell>
-        </row>
-        <row r="111">
-          <cell r="A111">
-            <v>401071</v>
-          </cell>
-          <cell r="T111" t="str">
-            <v>8970339891</v>
-          </cell>
-        </row>
-        <row r="112">
-          <cell r="A112">
-            <v>401072</v>
-          </cell>
-          <cell r="T112" t="str">
-            <v>8941010571</v>
-          </cell>
-        </row>
-        <row r="113">
-          <cell r="A113">
-            <v>401073</v>
-          </cell>
-          <cell r="T113" t="str">
-            <v>8973341070AA</v>
-          </cell>
-        </row>
-        <row r="114">
-          <cell r="A114">
-            <v>341074</v>
-          </cell>
-          <cell r="B114" t="str">
-            <v>14.4739.10</v>
-          </cell>
-          <cell r="T114" t="str">
-            <v>4243135060</v>
-          </cell>
-        </row>
-        <row r="115">
-          <cell r="A115">
-            <v>251075</v>
-          </cell>
-          <cell r="K115" t="str">
-            <v>AD1159</v>
-          </cell>
-          <cell r="L115" t="str">
-            <v>07050075</v>
-          </cell>
-          <cell r="M115" t="str">
-            <v>07050075</v>
-          </cell>
-          <cell r="T115" t="str">
-            <v>MK321338</v>
-          </cell>
-        </row>
-        <row r="116">
-          <cell r="A116">
-            <v>321081</v>
-          </cell>
-          <cell r="C116" t="str">
-            <v>DB4421</v>
-          </cell>
-          <cell r="H116" t="str">
-            <v>0 986 477 236</v>
-          </cell>
-          <cell r="R116" t="str">
-            <v>94037800</v>
-          </cell>
-          <cell r="S116"/>
-          <cell r="T116" t="str">
-            <v>4351165D00</v>
-          </cell>
-        </row>
-        <row r="117">
-          <cell r="A117">
-            <v>191082</v>
-          </cell>
-          <cell r="B117" t="str">
-            <v>14.7079.10</v>
-          </cell>
-          <cell r="C117" t="str">
-            <v>DB4307</v>
-          </cell>
-          <cell r="L117" t="str">
-            <v>07050087</v>
-          </cell>
-          <cell r="M117" t="str">
-            <v>07050087</v>
-          </cell>
-          <cell r="R117" t="str">
-            <v>94015600</v>
-          </cell>
-          <cell r="S117"/>
-          <cell r="T117" t="str">
-            <v>21080350207000</v>
-          </cell>
-        </row>
-        <row r="118">
-          <cell r="A118">
-            <v>341083</v>
-          </cell>
-          <cell r="S118" t="str">
-            <v>DN1217</v>
-          </cell>
-          <cell r="T118" t="str">
-            <v>4243137080</v>
-          </cell>
-        </row>
-        <row r="119">
-          <cell r="A119">
-            <v>341084</v>
-          </cell>
-          <cell r="S119" t="str">
-            <v>DN1226</v>
-          </cell>
-          <cell r="T119" t="str">
-            <v>4351236190</v>
-          </cell>
-        </row>
-        <row r="120">
-          <cell r="A120">
-            <v>131085</v>
-          </cell>
-          <cell r="B120" t="str">
-            <v>14.7098.20</v>
-          </cell>
-          <cell r="L120" t="str">
-            <v>07050076</v>
-          </cell>
-          <cell r="M120" t="str">
-            <v>07050076</v>
-          </cell>
-          <cell r="Q120" t="str">
-            <v>BSG 30-225-005</v>
-          </cell>
-          <cell r="T120" t="str">
-            <v>4146930</v>
-          </cell>
-        </row>
-        <row r="121">
-          <cell r="A121">
-            <v>131086</v>
-          </cell>
-          <cell r="K121" t="str">
-            <v>AD5110</v>
-          </cell>
-          <cell r="L121" t="str">
-            <v>07050093</v>
-          </cell>
-          <cell r="M121" t="str">
-            <v>07050093</v>
-          </cell>
-          <cell r="T121" t="str">
-            <v>R2X61126AAN</v>
-          </cell>
-        </row>
-        <row r="122">
-          <cell r="A122">
-            <v>341087</v>
-          </cell>
-          <cell r="B122" t="str">
-            <v>14.E277.10</v>
-          </cell>
-          <cell r="T122" t="str">
-            <v>424310D100</v>
-          </cell>
-        </row>
-        <row r="123">
-          <cell r="A123" t="str">
-            <v>30997B</v>
-          </cell>
-          <cell r="T123"/>
-        </row>
-        <row r="124">
-          <cell r="A124">
-            <v>251088</v>
-          </cell>
-          <cell r="T124" t="str">
-            <v>MC862229</v>
-          </cell>
-        </row>
-        <row r="125">
-          <cell r="A125">
-            <v>511089</v>
-          </cell>
-          <cell r="R125">
-            <v>94036400</v>
-          </cell>
-          <cell r="T125" t="str">
-            <v>42431B1011</v>
-          </cell>
-        </row>
-        <row r="126">
-          <cell r="A126">
-            <v>261090</v>
-          </cell>
-          <cell r="B126" t="str">
-            <v>14.5073.10</v>
-          </cell>
-          <cell r="T126" t="str">
-            <v>4320608G11</v>
-          </cell>
-        </row>
-        <row r="127">
-          <cell r="A127">
-            <v>261091</v>
-          </cell>
-          <cell r="R127" t="str">
-            <v>94026900</v>
-          </cell>
-          <cell r="S127"/>
-          <cell r="T127" t="str">
-            <v>432064M000</v>
-          </cell>
-        </row>
-        <row r="128">
-          <cell r="A128">
-            <v>341092</v>
-          </cell>
-          <cell r="R128" t="str">
-            <v>94045200</v>
-          </cell>
-          <cell r="S128"/>
-          <cell r="T128" t="str">
-            <v>424310D030000</v>
-          </cell>
-        </row>
-      </sheetData>
-      <sheetData sheetId="1"/>
-    </sheetDataSet>
-  </externalBook>
-</externalLink>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -14032,153 +10624,130 @@
       <c r="A2" s="3">
         <v>13275</v>
       </c>
-      <c r="B2" s="3" t="str">
-        <f>VLOOKUP(A:A,[1]Sheet1!$A:$T,20,0)</f>
-        <v>043860</v>
+      <c r="B2" s="3" t="s">
+        <v>679</v>
       </c>
     </row>
     <row r="3" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A3" s="3">
         <v>13278</v>
       </c>
-      <c r="B3" s="3" t="str">
-        <f>VLOOKUP(A:A,[1]Sheet1!$A:$T,20,0)</f>
-        <v>HST1126AB</v>
+      <c r="B3" s="3" t="s">
+        <v>680</v>
       </c>
     </row>
     <row r="4" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A4" s="3">
         <v>13284</v>
       </c>
-      <c r="B4" s="3" t="str">
-        <f>VLOOKUP(A:A,[1]Sheet1!$A:$T,20,0)</f>
-        <v>90PY1126</v>
+      <c r="B4" s="3" t="s">
+        <v>681</v>
       </c>
     </row>
     <row r="5" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A5" s="3">
         <v>45387</v>
       </c>
-      <c r="B5" s="3" t="str">
-        <f>VLOOKUP(A:A,[1]Sheet1!$A:$T,20,0)</f>
-        <v>3757089</v>
+      <c r="B5" s="3" t="s">
+        <v>682</v>
       </c>
     </row>
     <row r="6" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A6" s="3">
         <v>45396</v>
       </c>
-      <c r="B6" s="3" t="str">
-        <f>VLOOKUP(A:A,[1]Sheet1!$A:$T,20,0)</f>
-        <v>28288</v>
+      <c r="B6" s="3" t="s">
+        <v>683</v>
       </c>
     </row>
     <row r="7" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A7" s="3" t="s">
         <v>195</v>
       </c>
-      <c r="B7" s="3" t="str">
-        <f>VLOOKUP(A:A,[1]Sheet1!$A:$T,20,0)</f>
-        <v>2952956</v>
+      <c r="B7" s="3" t="s">
+        <v>684</v>
       </c>
     </row>
     <row r="8" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A8" s="3">
         <v>45473</v>
       </c>
-      <c r="B8" s="3">
-        <f>VLOOKUP(A:A,[1]Sheet1!$A:$T,20,0)</f>
-        <v>0</v>
-      </c>
+      <c r="B8" s="3"/>
     </row>
     <row r="9" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A9" s="3">
         <v>59480</v>
       </c>
-      <c r="B9" s="3" t="str">
-        <f>VLOOKUP(A:A,[1]Sheet1!$A:$T,20,0)</f>
-        <v>57RS305352</v>
+      <c r="B9" s="3" t="s">
+        <v>685</v>
       </c>
     </row>
     <row r="10" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A10" s="3">
         <v>37737</v>
       </c>
-      <c r="B10" s="3">
-        <f>VLOOKUP(A:A,[1]Sheet1!$A:$T,20,0)</f>
-        <v>0</v>
-      </c>
+      <c r="B10" s="3"/>
     </row>
     <row r="11" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A11" s="3" t="s">
         <v>229</v>
       </c>
-      <c r="B11" s="3" t="str">
-        <f>VLOOKUP(A:A,[1]Sheet1!$A:$T,20,0)</f>
-        <v>3757089</v>
+      <c r="B11" s="3" t="s">
+        <v>682</v>
       </c>
     </row>
     <row r="12" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A12" s="3">
         <v>63999</v>
       </c>
-      <c r="B12" s="3" t="str">
-        <f>VLOOKUP(A:A,[1]Sheet1!$A:$T,20,0)</f>
-        <v>3302350207001</v>
+      <c r="B12" s="3" t="s">
+        <v>686</v>
       </c>
     </row>
     <row r="13" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A13" s="3">
         <v>251070</v>
       </c>
-      <c r="B13" s="3" t="str">
-        <f>VLOOKUP(A:A,[1]Sheet1!$A:$T,20,0)</f>
-        <v>MC862229</v>
+      <c r="B13" s="3" t="s">
+        <v>687</v>
       </c>
     </row>
     <row r="14" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A14" s="3">
         <v>401072</v>
       </c>
-      <c r="B14" s="3" t="str">
-        <f>VLOOKUP(A:A,[1]Sheet1!$A:$T,20,0)</f>
-        <v>8941010571</v>
+      <c r="B14" s="3" t="s">
+        <v>688</v>
       </c>
     </row>
     <row r="15" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A15" s="3">
         <v>401073</v>
       </c>
-      <c r="B15" s="3" t="str">
-        <f>VLOOKUP(A:A,[1]Sheet1!$A:$T,20,0)</f>
-        <v>8973341070AA</v>
+      <c r="B15" s="3" t="s">
+        <v>689</v>
       </c>
     </row>
     <row r="16" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A16" s="3">
         <v>131086</v>
       </c>
-      <c r="B16" s="3" t="str">
-        <f>VLOOKUP(A:A,[1]Sheet1!$A:$T,20,0)</f>
-        <v>R2X61126AAN</v>
+      <c r="B16" s="3" t="s">
+        <v>690</v>
       </c>
     </row>
     <row r="17" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A17" s="3" t="s">
         <v>233</v>
       </c>
-      <c r="B17" s="3">
-        <f>VLOOKUP(A:A,[1]Sheet1!$A:$T,20,0)</f>
-        <v>0</v>
-      </c>
+      <c r="B17" s="3"/>
     </row>
     <row r="18" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A18" s="3">
         <v>251088</v>
       </c>
-      <c r="B18" s="3" t="str">
-        <f>VLOOKUP(A:A,[1]Sheet1!$A:$T,20,0)</f>
-        <v>MC862229</v>
+      <c r="B18" s="3" t="s">
+        <v>687</v>
       </c>
     </row>
     <row r="19" spans="1:3" x14ac:dyDescent="0.3">

</xml_diff>